<commit_message>
feat(fb-groups): sync 5 groups post results, update Notion DBs, post history & top 5 recommendations
</commit_message>
<xml_diff>
--- a/song_anh_seo_keywords_historical_database.xlsx
+++ b/song_anh_seo_keywords_historical_database.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I683"/>
+  <dimension ref="A1:I705"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -27061,6 +27061,864 @@
         </is>
       </c>
     </row>
+    <row r="684">
+      <c r="A684" t="inlineStr">
+        <is>
+          <t>21/08/2026</t>
+        </is>
+      </c>
+      <c r="B684" t="n">
+        <v>1</v>
+      </c>
+      <c r="C684" t="inlineStr">
+        <is>
+          <t>mô hình quy hoạch</t>
+        </is>
+      </c>
+      <c r="D684" t="n">
+        <v>6.5</v>
+      </c>
+      <c r="E684" t="n">
+        <v>43</v>
+      </c>
+      <c r="F684" t="n">
+        <v>3</v>
+      </c>
+      <c r="G684" t="inlineStr">
+        <is>
+          <t>6.98%</t>
+        </is>
+      </c>
+      <c r="H684" t="inlineStr">
+        <is>
+          <t>https://mohinhkientruc.org/danh-muc-du-an/mo-hinh-quy-hoach/</t>
+        </is>
+      </c>
+      <c r="I684" t="inlineStr">
+        <is>
+          <t>🖼️ Image Pack</t>
+        </is>
+      </c>
+    </row>
+    <row r="685">
+      <c r="A685" t="inlineStr">
+        <is>
+          <t>21/08/2026</t>
+        </is>
+      </c>
+      <c r="B685" t="n">
+        <v>2</v>
+      </c>
+      <c r="C685" t="inlineStr">
+        <is>
+          <t>mô hình kiến trúc</t>
+        </is>
+      </c>
+      <c r="D685" t="n">
+        <v>18.5</v>
+      </c>
+      <c r="E685" t="n">
+        <v>88</v>
+      </c>
+      <c r="F685" t="n">
+        <v>4</v>
+      </c>
+      <c r="G685" t="inlineStr">
+        <is>
+          <t>4.55%</t>
+        </is>
+      </c>
+      <c r="H685" t="inlineStr">
+        <is>
+          <t>https://mohinhkientruc.org/mo-hinh-kien-truc/</t>
+        </is>
+      </c>
+      <c r="I685" t="inlineStr">
+        <is>
+          <t>Standard Snippet</t>
+        </is>
+      </c>
+    </row>
+    <row r="686">
+      <c r="A686" t="inlineStr">
+        <is>
+          <t>21/08/2026</t>
+        </is>
+      </c>
+      <c r="B686" t="n">
+        <v>3</v>
+      </c>
+      <c r="C686" t="inlineStr">
+        <is>
+          <t>mô hình cao tầng</t>
+        </is>
+      </c>
+      <c r="D686" t="n">
+        <v>5</v>
+      </c>
+      <c r="E686" t="n">
+        <v>980</v>
+      </c>
+      <c r="F686" t="n">
+        <v>54</v>
+      </c>
+      <c r="G686" t="inlineStr">
+        <is>
+          <t>5.51%</t>
+        </is>
+      </c>
+      <c r="H686" t="inlineStr">
+        <is>
+          <t>https://mohinhkientruc.org/sa-ban-cao-tang/</t>
+        </is>
+      </c>
+      <c r="I686" t="inlineStr">
+        <is>
+          <t>Standard Snippet</t>
+        </is>
+      </c>
+    </row>
+    <row r="687">
+      <c r="A687" t="inlineStr">
+        <is>
+          <t>21/08/2026</t>
+        </is>
+      </c>
+      <c r="B687" t="n">
+        <v>4</v>
+      </c>
+      <c r="C687" t="inlineStr">
+        <is>
+          <t>mô hình nhà máy</t>
+        </is>
+      </c>
+      <c r="D687" t="n">
+        <v>6</v>
+      </c>
+      <c r="E687" t="n">
+        <v>1120</v>
+      </c>
+      <c r="F687" t="n">
+        <v>68</v>
+      </c>
+      <c r="G687" t="inlineStr">
+        <is>
+          <t>6.07%</t>
+        </is>
+      </c>
+      <c r="H687" t="inlineStr">
+        <is>
+          <t>https://mohinhkientruc.org/mo-hinh-nha-may/</t>
+        </is>
+      </c>
+      <c r="I687" t="inlineStr">
+        <is>
+          <t>Standard Snippet</t>
+        </is>
+      </c>
+    </row>
+    <row r="688">
+      <c r="A688" t="inlineStr">
+        <is>
+          <t>21/08/2026</t>
+        </is>
+      </c>
+      <c r="B688" t="n">
+        <v>5</v>
+      </c>
+      <c r="C688" t="inlineStr">
+        <is>
+          <t>mô hình thiết bị</t>
+        </is>
+      </c>
+      <c r="D688" t="n">
+        <v>9</v>
+      </c>
+      <c r="E688" t="n">
+        <v>640</v>
+      </c>
+      <c r="F688" t="n">
+        <v>25</v>
+      </c>
+      <c r="G688" t="inlineStr">
+        <is>
+          <t>3.91%</t>
+        </is>
+      </c>
+      <c r="H688" t="inlineStr">
+        <is>
+          <t>https://mohinhkientruc.org/mo-hinh-3d/</t>
+        </is>
+      </c>
+      <c r="I688" t="inlineStr">
+        <is>
+          <t>Standard Snippet</t>
+        </is>
+      </c>
+    </row>
+    <row r="689">
+      <c r="A689" t="inlineStr">
+        <is>
+          <t>21/08/2026</t>
+        </is>
+      </c>
+      <c r="B689" t="n">
+        <v>6</v>
+      </c>
+      <c r="C689" t="inlineStr">
+        <is>
+          <t>mô hình trường học</t>
+        </is>
+      </c>
+      <c r="D689" t="n">
+        <v>7</v>
+      </c>
+      <c r="E689" t="n">
+        <v>720</v>
+      </c>
+      <c r="F689" t="n">
+        <v>38</v>
+      </c>
+      <c r="G689" t="inlineStr">
+        <is>
+          <t>5.28%</t>
+        </is>
+      </c>
+      <c r="H689" t="inlineStr">
+        <is>
+          <t>https://mohinhkientruc.org/lam-sa-ban-truong-hoc/</t>
+        </is>
+      </c>
+      <c r="I689" t="inlineStr">
+        <is>
+          <t>Standard Snippet</t>
+        </is>
+      </c>
+    </row>
+    <row r="690">
+      <c r="A690" t="inlineStr">
+        <is>
+          <t>21/08/2026</t>
+        </is>
+      </c>
+      <c r="B690" t="n">
+        <v>7</v>
+      </c>
+      <c r="C690" t="inlineStr">
+        <is>
+          <t>mô hình bệnh viện</t>
+        </is>
+      </c>
+      <c r="D690" t="n">
+        <v>8</v>
+      </c>
+      <c r="E690" t="n">
+        <v>530</v>
+      </c>
+      <c r="F690" t="n">
+        <v>22</v>
+      </c>
+      <c r="G690" t="inlineStr">
+        <is>
+          <t>4.15%</t>
+        </is>
+      </c>
+      <c r="H690" t="inlineStr">
+        <is>
+          <t>https://mohinhkientruc.org/mo-hinh-tod-sa-ban/</t>
+        </is>
+      </c>
+      <c r="I690" t="inlineStr">
+        <is>
+          <t>Standard Snippet</t>
+        </is>
+      </c>
+    </row>
+    <row r="691">
+      <c r="A691" t="inlineStr">
+        <is>
+          <t>21/08/2026</t>
+        </is>
+      </c>
+      <c r="B691" t="n">
+        <v>8</v>
+      </c>
+      <c r="C691" t="inlineStr">
+        <is>
+          <t>sa bàn quy hoạch</t>
+        </is>
+      </c>
+      <c r="D691" t="n">
+        <v>4</v>
+      </c>
+      <c r="E691" t="n">
+        <v>1650</v>
+      </c>
+      <c r="F691" t="n">
+        <v>118</v>
+      </c>
+      <c r="G691" t="inlineStr">
+        <is>
+          <t>7.15%</t>
+        </is>
+      </c>
+      <c r="H691" t="inlineStr">
+        <is>
+          <t>https://mohinhkientruc.org/dich-vu-lam-sa-ban-quy-hoach/</t>
+        </is>
+      </c>
+      <c r="I691" t="inlineStr">
+        <is>
+          <t>🖼️ Image Pack</t>
+        </is>
+      </c>
+    </row>
+    <row r="692">
+      <c r="A692" t="inlineStr">
+        <is>
+          <t>21/08/2026</t>
+        </is>
+      </c>
+      <c r="B692" t="n">
+        <v>9</v>
+      </c>
+      <c r="C692" t="inlineStr">
+        <is>
+          <t>sa bàn kiến trúc</t>
+        </is>
+      </c>
+      <c r="D692" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="E692" t="n">
+        <v>2100</v>
+      </c>
+      <c r="F692" t="n">
+        <v>135</v>
+      </c>
+      <c r="G692" t="inlineStr">
+        <is>
+          <t>6.43%</t>
+        </is>
+      </c>
+      <c r="H692" t="inlineStr">
+        <is>
+          <t>https://mohinhkientruc.org/sa-ban-kien-truc/</t>
+        </is>
+      </c>
+      <c r="I692" t="inlineStr">
+        <is>
+          <t>Standard Snippet</t>
+        </is>
+      </c>
+    </row>
+    <row r="693">
+      <c r="A693" t="inlineStr">
+        <is>
+          <t>21/08/2026</t>
+        </is>
+      </c>
+      <c r="B693" t="n">
+        <v>10</v>
+      </c>
+      <c r="C693" t="inlineStr">
+        <is>
+          <t>sa bàn cao tầng</t>
+        </is>
+      </c>
+      <c r="D693" t="n">
+        <v>5.5</v>
+      </c>
+      <c r="E693" t="n">
+        <v>870</v>
+      </c>
+      <c r="F693" t="n">
+        <v>46</v>
+      </c>
+      <c r="G693" t="inlineStr">
+        <is>
+          <t>5.29%</t>
+        </is>
+      </c>
+      <c r="H693" t="inlineStr">
+        <is>
+          <t>https://mohinhkientruc.org/sa-ban-cao-tang/</t>
+        </is>
+      </c>
+      <c r="I693" t="inlineStr">
+        <is>
+          <t>Standard Snippet</t>
+        </is>
+      </c>
+    </row>
+    <row r="694">
+      <c r="A694" t="inlineStr">
+        <is>
+          <t>21/08/2026</t>
+        </is>
+      </c>
+      <c r="B694" t="n">
+        <v>11</v>
+      </c>
+      <c r="C694" t="inlineStr">
+        <is>
+          <t>sa bàn nhà máy</t>
+        </is>
+      </c>
+      <c r="D694" t="n">
+        <v>6.5</v>
+      </c>
+      <c r="E694" t="n">
+        <v>940</v>
+      </c>
+      <c r="F694" t="n">
+        <v>52</v>
+      </c>
+      <c r="G694" t="inlineStr">
+        <is>
+          <t>5.53%</t>
+        </is>
+      </c>
+      <c r="H694" t="inlineStr">
+        <is>
+          <t>https://mohinhkientruc.org/thi-cong-sa-ban-nha-may-khu-cong-nghiep/</t>
+        </is>
+      </c>
+      <c r="I694" t="inlineStr">
+        <is>
+          <t>Standard Snippet</t>
+        </is>
+      </c>
+    </row>
+    <row r="695">
+      <c r="A695" t="inlineStr">
+        <is>
+          <t>21/08/2026</t>
+        </is>
+      </c>
+      <c r="B695" t="n">
+        <v>12</v>
+      </c>
+      <c r="C695" t="inlineStr">
+        <is>
+          <t>sa bàn thiết bị</t>
+        </is>
+      </c>
+      <c r="D695" t="n">
+        <v>9.5</v>
+      </c>
+      <c r="E695" t="n">
+        <v>480</v>
+      </c>
+      <c r="F695" t="n">
+        <v>18</v>
+      </c>
+      <c r="G695" t="inlineStr">
+        <is>
+          <t>3.75%</t>
+        </is>
+      </c>
+      <c r="H695" t="inlineStr">
+        <is>
+          <t>https://mohinhkientruc.org/sa-ban-noi-that/</t>
+        </is>
+      </c>
+      <c r="I695" t="inlineStr">
+        <is>
+          <t>Standard Snippet</t>
+        </is>
+      </c>
+    </row>
+    <row r="696">
+      <c r="A696" t="inlineStr">
+        <is>
+          <t>21/08/2026</t>
+        </is>
+      </c>
+      <c r="B696" t="n">
+        <v>13</v>
+      </c>
+      <c r="C696" t="inlineStr">
+        <is>
+          <t>sa bàn trường học</t>
+        </is>
+      </c>
+      <c r="D696" t="n">
+        <v>8.5</v>
+      </c>
+      <c r="E696" t="n">
+        <v>2</v>
+      </c>
+      <c r="F696" t="n">
+        <v>1</v>
+      </c>
+      <c r="G696" t="inlineStr">
+        <is>
+          <t>50.00%</t>
+        </is>
+      </c>
+      <c r="H696" t="inlineStr">
+        <is>
+          <t>https://mohinhkientruc.org/lam-sa-ban-truong-hoc/</t>
+        </is>
+      </c>
+      <c r="I696" t="inlineStr">
+        <is>
+          <t>Standard Snippet</t>
+        </is>
+      </c>
+    </row>
+    <row r="697">
+      <c r="A697" t="inlineStr">
+        <is>
+          <t>21/08/2026</t>
+        </is>
+      </c>
+      <c r="B697" t="n">
+        <v>14</v>
+      </c>
+      <c r="C697" t="inlineStr">
+        <is>
+          <t>sa bàn bệnh viện</t>
+        </is>
+      </c>
+      <c r="D697" t="n">
+        <v>8.5</v>
+      </c>
+      <c r="E697" t="n">
+        <v>590</v>
+      </c>
+      <c r="F697" t="n">
+        <v>26</v>
+      </c>
+      <c r="G697" t="inlineStr">
+        <is>
+          <t>4.41%</t>
+        </is>
+      </c>
+      <c r="H697" t="inlineStr">
+        <is>
+          <t>https://mohinhkientruc.org/du-an-noi-bat/</t>
+        </is>
+      </c>
+      <c r="I697" t="inlineStr">
+        <is>
+          <t>Standard Snippet</t>
+        </is>
+      </c>
+    </row>
+    <row r="698">
+      <c r="A698" t="inlineStr">
+        <is>
+          <t>21/08/2026</t>
+        </is>
+      </c>
+      <c r="B698" t="n">
+        <v>15</v>
+      </c>
+      <c r="C698" t="inlineStr">
+        <is>
+          <t>vận chuyển mô hình</t>
+        </is>
+      </c>
+      <c r="D698" t="n">
+        <v>6.8</v>
+      </c>
+      <c r="E698" t="n">
+        <v>820</v>
+      </c>
+      <c r="F698" t="n">
+        <v>45</v>
+      </c>
+      <c r="G698" t="inlineStr">
+        <is>
+          <t>5.49%</t>
+        </is>
+      </c>
+      <c r="H698" t="inlineStr">
+        <is>
+          <t>https://mohinhkientruc.org/van-chuyen-sa-ban-kien-truc/</t>
+        </is>
+      </c>
+      <c r="I698" t="inlineStr">
+        <is>
+          <t>Standard Snippet</t>
+        </is>
+      </c>
+    </row>
+    <row r="699">
+      <c r="A699" t="inlineStr">
+        <is>
+          <t>21/08/2026</t>
+        </is>
+      </c>
+      <c r="B699" t="n">
+        <v>16</v>
+      </c>
+      <c r="C699" t="inlineStr">
+        <is>
+          <t>vận chuyển sa bàn</t>
+        </is>
+      </c>
+      <c r="D699" t="n">
+        <v>7.2</v>
+      </c>
+      <c r="E699" t="n">
+        <v>760</v>
+      </c>
+      <c r="F699" t="n">
+        <v>38</v>
+      </c>
+      <c r="G699" t="inlineStr">
+        <is>
+          <t>5.00%</t>
+        </is>
+      </c>
+      <c r="H699" t="inlineStr">
+        <is>
+          <t>https://mohinhkientruc.org/van-chuyen-sa-ban-kien-truc/</t>
+        </is>
+      </c>
+      <c r="I699" t="inlineStr">
+        <is>
+          <t>Standard Snippet</t>
+        </is>
+      </c>
+    </row>
+    <row r="700">
+      <c r="A700" t="inlineStr">
+        <is>
+          <t>21/08/2026</t>
+        </is>
+      </c>
+      <c r="B700" t="n">
+        <v>17</v>
+      </c>
+      <c r="C700" t="inlineStr">
+        <is>
+          <t>sửa chữa mô hình</t>
+        </is>
+      </c>
+      <c r="D700" t="n">
+        <v>5.4</v>
+      </c>
+      <c r="E700" t="n">
+        <v>930</v>
+      </c>
+      <c r="F700" t="n">
+        <v>58</v>
+      </c>
+      <c r="G700" t="inlineStr">
+        <is>
+          <t>6.24%</t>
+        </is>
+      </c>
+      <c r="H700" t="inlineStr">
+        <is>
+          <t>https://mohinhkientruc.org/sua-chua-mo-hinh-kien-truc/</t>
+        </is>
+      </c>
+      <c r="I700" t="inlineStr">
+        <is>
+          <t>Standard Snippet</t>
+        </is>
+      </c>
+    </row>
+    <row r="701">
+      <c r="A701" t="inlineStr">
+        <is>
+          <t>21/08/2026</t>
+        </is>
+      </c>
+      <c r="B701" t="n">
+        <v>18</v>
+      </c>
+      <c r="C701" t="inlineStr">
+        <is>
+          <t>sửa chữa sa bàn</t>
+        </is>
+      </c>
+      <c r="D701" t="n">
+        <v>5.8</v>
+      </c>
+      <c r="E701" t="n">
+        <v>880</v>
+      </c>
+      <c r="F701" t="n">
+        <v>52</v>
+      </c>
+      <c r="G701" t="inlineStr">
+        <is>
+          <t>5.91%</t>
+        </is>
+      </c>
+      <c r="H701" t="inlineStr">
+        <is>
+          <t>https://mohinhkientruc.org/sua-chua-mo-hinh-kien-truc/</t>
+        </is>
+      </c>
+      <c r="I701" t="inlineStr">
+        <is>
+          <t>Standard Snippet</t>
+        </is>
+      </c>
+    </row>
+    <row r="702">
+      <c r="A702" t="inlineStr">
+        <is>
+          <t>21/08/2026</t>
+        </is>
+      </c>
+      <c r="B702" t="n">
+        <v>19</v>
+      </c>
+      <c r="C702" t="inlineStr">
+        <is>
+          <t>công ty mô hình kiến trúc</t>
+        </is>
+      </c>
+      <c r="D702" t="n">
+        <v>45</v>
+      </c>
+      <c r="E702" t="n">
+        <v>24</v>
+      </c>
+      <c r="F702" t="n">
+        <v>0</v>
+      </c>
+      <c r="G702" t="inlineStr">
+        <is>
+          <t>0.00%</t>
+        </is>
+      </c>
+      <c r="H702" t="inlineStr">
+        <is>
+          <t>https://mohinhkientruc.org/cong-ty-lam-mo-hinh/</t>
+        </is>
+      </c>
+      <c r="I702" t="inlineStr">
+        <is>
+          <t>🖼️ Image Pack</t>
+        </is>
+      </c>
+    </row>
+    <row r="703">
+      <c r="A703" t="inlineStr">
+        <is>
+          <t>21/08/2026</t>
+        </is>
+      </c>
+      <c r="B703" t="n">
+        <v>20</v>
+      </c>
+      <c r="C703" t="inlineStr">
+        <is>
+          <t>công ty sa bàn kiến trúc</t>
+        </is>
+      </c>
+      <c r="D703" t="n">
+        <v>3.2</v>
+      </c>
+      <c r="E703" t="n">
+        <v>2410</v>
+      </c>
+      <c r="F703" t="n">
+        <v>168</v>
+      </c>
+      <c r="G703" t="inlineStr">
+        <is>
+          <t>6.97%</t>
+        </is>
+      </c>
+      <c r="H703" t="inlineStr">
+        <is>
+          <t>https://mohinhkientruc.org/</t>
+        </is>
+      </c>
+      <c r="I703" t="inlineStr">
+        <is>
+          <t>Standard Snippet</t>
+        </is>
+      </c>
+    </row>
+    <row r="704">
+      <c r="A704" t="inlineStr">
+        <is>
+          <t>21/08/2026</t>
+        </is>
+      </c>
+      <c r="B704" t="n">
+        <v>21</v>
+      </c>
+      <c r="C704" t="inlineStr">
+        <is>
+          <t>làm mô hình</t>
+        </is>
+      </c>
+      <c r="D704" t="n">
+        <v>4.2</v>
+      </c>
+      <c r="E704" t="n">
+        <v>1780</v>
+      </c>
+      <c r="F704" t="n">
+        <v>121</v>
+      </c>
+      <c r="G704" t="inlineStr">
+        <is>
+          <t>6.80%</t>
+        </is>
+      </c>
+      <c r="H704" t="inlineStr">
+        <is>
+          <t>https://mohinhkientruc.org/lam-mo-hinh-kien-truc/</t>
+        </is>
+      </c>
+      <c r="I704" t="inlineStr">
+        <is>
+          <t>Standard Snippet</t>
+        </is>
+      </c>
+    </row>
+    <row r="705">
+      <c r="A705" t="inlineStr">
+        <is>
+          <t>21/08/2026</t>
+        </is>
+      </c>
+      <c r="B705" t="n">
+        <v>22</v>
+      </c>
+      <c r="C705" t="inlineStr">
+        <is>
+          <t>làm sa bàn</t>
+        </is>
+      </c>
+      <c r="D705" t="n">
+        <v>4.6</v>
+      </c>
+      <c r="E705" t="n">
+        <v>1620</v>
+      </c>
+      <c r="F705" t="n">
+        <v>104</v>
+      </c>
+      <c r="G705" t="inlineStr">
+        <is>
+          <t>6.42%</t>
+        </is>
+      </c>
+      <c r="H705" t="inlineStr">
+        <is>
+          <t>https://mohinhkientruc.org/lam-sa-ban/</t>
+        </is>
+      </c>
+      <c r="I705" t="inlineStr">
+        <is>
+          <t>Standard Snippet</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat(ui): optimize webapp layout with clean icons and keyword badges, reducing dense text
</commit_message>
<xml_diff>
--- a/song_anh_seo_keywords_historical_database.xlsx
+++ b/song_anh_seo_keywords_historical_database.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I705"/>
+  <dimension ref="A1:I727"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -27919,6 +27919,864 @@
         </is>
       </c>
     </row>
+    <row r="706">
+      <c r="A706" t="inlineStr">
+        <is>
+          <t>23/08/2026</t>
+        </is>
+      </c>
+      <c r="B706" t="n">
+        <v>1</v>
+      </c>
+      <c r="C706" t="inlineStr">
+        <is>
+          <t>mô hình quy hoạch</t>
+        </is>
+      </c>
+      <c r="D706" t="n">
+        <v>6.8</v>
+      </c>
+      <c r="E706" t="n">
+        <v>46</v>
+      </c>
+      <c r="F706" t="n">
+        <v>3</v>
+      </c>
+      <c r="G706" t="inlineStr">
+        <is>
+          <t>6.52%</t>
+        </is>
+      </c>
+      <c r="H706" t="inlineStr">
+        <is>
+          <t>https://mohinhkientruc.org/danh-muc-du-an/mo-hinh-quy-hoach/</t>
+        </is>
+      </c>
+      <c r="I706" t="inlineStr">
+        <is>
+          <t>🖼️ Image Pack</t>
+        </is>
+      </c>
+    </row>
+    <row r="707">
+      <c r="A707" t="inlineStr">
+        <is>
+          <t>23/08/2026</t>
+        </is>
+      </c>
+      <c r="B707" t="n">
+        <v>2</v>
+      </c>
+      <c r="C707" t="inlineStr">
+        <is>
+          <t>mô hình kiến trúc</t>
+        </is>
+      </c>
+      <c r="D707" t="n">
+        <v>18.3</v>
+      </c>
+      <c r="E707" t="n">
+        <v>108</v>
+      </c>
+      <c r="F707" t="n">
+        <v>4</v>
+      </c>
+      <c r="G707" t="inlineStr">
+        <is>
+          <t>3.70%</t>
+        </is>
+      </c>
+      <c r="H707" t="inlineStr">
+        <is>
+          <t>https://mohinhkientruc.org/mo-hinh-kien-truc/</t>
+        </is>
+      </c>
+      <c r="I707" t="inlineStr">
+        <is>
+          <t>Standard Snippet</t>
+        </is>
+      </c>
+    </row>
+    <row r="708">
+      <c r="A708" t="inlineStr">
+        <is>
+          <t>23/08/2026</t>
+        </is>
+      </c>
+      <c r="B708" t="n">
+        <v>3</v>
+      </c>
+      <c r="C708" t="inlineStr">
+        <is>
+          <t>mô hình cao tầng</t>
+        </is>
+      </c>
+      <c r="D708" t="n">
+        <v>5</v>
+      </c>
+      <c r="E708" t="n">
+        <v>980</v>
+      </c>
+      <c r="F708" t="n">
+        <v>54</v>
+      </c>
+      <c r="G708" t="inlineStr">
+        <is>
+          <t>5.51%</t>
+        </is>
+      </c>
+      <c r="H708" t="inlineStr">
+        <is>
+          <t>https://mohinhkientruc.org/sa-ban-cao-tang/</t>
+        </is>
+      </c>
+      <c r="I708" t="inlineStr">
+        <is>
+          <t>Standard Snippet</t>
+        </is>
+      </c>
+    </row>
+    <row r="709">
+      <c r="A709" t="inlineStr">
+        <is>
+          <t>23/08/2026</t>
+        </is>
+      </c>
+      <c r="B709" t="n">
+        <v>4</v>
+      </c>
+      <c r="C709" t="inlineStr">
+        <is>
+          <t>mô hình nhà máy</t>
+        </is>
+      </c>
+      <c r="D709" t="n">
+        <v>6</v>
+      </c>
+      <c r="E709" t="n">
+        <v>1120</v>
+      </c>
+      <c r="F709" t="n">
+        <v>68</v>
+      </c>
+      <c r="G709" t="inlineStr">
+        <is>
+          <t>6.07%</t>
+        </is>
+      </c>
+      <c r="H709" t="inlineStr">
+        <is>
+          <t>https://mohinhkientruc.org/mo-hinh-nha-may/</t>
+        </is>
+      </c>
+      <c r="I709" t="inlineStr">
+        <is>
+          <t>Standard Snippet</t>
+        </is>
+      </c>
+    </row>
+    <row r="710">
+      <c r="A710" t="inlineStr">
+        <is>
+          <t>23/08/2026</t>
+        </is>
+      </c>
+      <c r="B710" t="n">
+        <v>5</v>
+      </c>
+      <c r="C710" t="inlineStr">
+        <is>
+          <t>mô hình thiết bị</t>
+        </is>
+      </c>
+      <c r="D710" t="n">
+        <v>9</v>
+      </c>
+      <c r="E710" t="n">
+        <v>640</v>
+      </c>
+      <c r="F710" t="n">
+        <v>25</v>
+      </c>
+      <c r="G710" t="inlineStr">
+        <is>
+          <t>3.91%</t>
+        </is>
+      </c>
+      <c r="H710" t="inlineStr">
+        <is>
+          <t>https://mohinhkientruc.org/mo-hinh-3d/</t>
+        </is>
+      </c>
+      <c r="I710" t="inlineStr">
+        <is>
+          <t>Standard Snippet</t>
+        </is>
+      </c>
+    </row>
+    <row r="711">
+      <c r="A711" t="inlineStr">
+        <is>
+          <t>23/08/2026</t>
+        </is>
+      </c>
+      <c r="B711" t="n">
+        <v>6</v>
+      </c>
+      <c r="C711" t="inlineStr">
+        <is>
+          <t>mô hình trường học</t>
+        </is>
+      </c>
+      <c r="D711" t="n">
+        <v>7</v>
+      </c>
+      <c r="E711" t="n">
+        <v>720</v>
+      </c>
+      <c r="F711" t="n">
+        <v>38</v>
+      </c>
+      <c r="G711" t="inlineStr">
+        <is>
+          <t>5.28%</t>
+        </is>
+      </c>
+      <c r="H711" t="inlineStr">
+        <is>
+          <t>https://mohinhkientruc.org/lam-sa-ban-truong-hoc/</t>
+        </is>
+      </c>
+      <c r="I711" t="inlineStr">
+        <is>
+          <t>Standard Snippet</t>
+        </is>
+      </c>
+    </row>
+    <row r="712">
+      <c r="A712" t="inlineStr">
+        <is>
+          <t>23/08/2026</t>
+        </is>
+      </c>
+      <c r="B712" t="n">
+        <v>7</v>
+      </c>
+      <c r="C712" t="inlineStr">
+        <is>
+          <t>mô hình bệnh viện</t>
+        </is>
+      </c>
+      <c r="D712" t="n">
+        <v>8</v>
+      </c>
+      <c r="E712" t="n">
+        <v>530</v>
+      </c>
+      <c r="F712" t="n">
+        <v>22</v>
+      </c>
+      <c r="G712" t="inlineStr">
+        <is>
+          <t>4.15%</t>
+        </is>
+      </c>
+      <c r="H712" t="inlineStr">
+        <is>
+          <t>https://mohinhkientruc.org/mo-hinh-tod-sa-ban/</t>
+        </is>
+      </c>
+      <c r="I712" t="inlineStr">
+        <is>
+          <t>Standard Snippet</t>
+        </is>
+      </c>
+    </row>
+    <row r="713">
+      <c r="A713" t="inlineStr">
+        <is>
+          <t>23/08/2026</t>
+        </is>
+      </c>
+      <c r="B713" t="n">
+        <v>8</v>
+      </c>
+      <c r="C713" t="inlineStr">
+        <is>
+          <t>sa bàn quy hoạch</t>
+        </is>
+      </c>
+      <c r="D713" t="n">
+        <v>4</v>
+      </c>
+      <c r="E713" t="n">
+        <v>1650</v>
+      </c>
+      <c r="F713" t="n">
+        <v>118</v>
+      </c>
+      <c r="G713" t="inlineStr">
+        <is>
+          <t>7.15%</t>
+        </is>
+      </c>
+      <c r="H713" t="inlineStr">
+        <is>
+          <t>https://mohinhkientruc.org/dich-vu-lam-sa-ban-quy-hoach/</t>
+        </is>
+      </c>
+      <c r="I713" t="inlineStr">
+        <is>
+          <t>🖼️ Image Pack</t>
+        </is>
+      </c>
+    </row>
+    <row r="714">
+      <c r="A714" t="inlineStr">
+        <is>
+          <t>23/08/2026</t>
+        </is>
+      </c>
+      <c r="B714" t="n">
+        <v>9</v>
+      </c>
+      <c r="C714" t="inlineStr">
+        <is>
+          <t>sa bàn kiến trúc</t>
+        </is>
+      </c>
+      <c r="D714" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="E714" t="n">
+        <v>2100</v>
+      </c>
+      <c r="F714" t="n">
+        <v>135</v>
+      </c>
+      <c r="G714" t="inlineStr">
+        <is>
+          <t>6.43%</t>
+        </is>
+      </c>
+      <c r="H714" t="inlineStr">
+        <is>
+          <t>https://mohinhkientruc.org/sa-ban-kien-truc/</t>
+        </is>
+      </c>
+      <c r="I714" t="inlineStr">
+        <is>
+          <t>Standard Snippet</t>
+        </is>
+      </c>
+    </row>
+    <row r="715">
+      <c r="A715" t="inlineStr">
+        <is>
+          <t>23/08/2026</t>
+        </is>
+      </c>
+      <c r="B715" t="n">
+        <v>10</v>
+      </c>
+      <c r="C715" t="inlineStr">
+        <is>
+          <t>sa bàn cao tầng</t>
+        </is>
+      </c>
+      <c r="D715" t="n">
+        <v>5.5</v>
+      </c>
+      <c r="E715" t="n">
+        <v>870</v>
+      </c>
+      <c r="F715" t="n">
+        <v>46</v>
+      </c>
+      <c r="G715" t="inlineStr">
+        <is>
+          <t>5.29%</t>
+        </is>
+      </c>
+      <c r="H715" t="inlineStr">
+        <is>
+          <t>https://mohinhkientruc.org/sa-ban-cao-tang/</t>
+        </is>
+      </c>
+      <c r="I715" t="inlineStr">
+        <is>
+          <t>Standard Snippet</t>
+        </is>
+      </c>
+    </row>
+    <row r="716">
+      <c r="A716" t="inlineStr">
+        <is>
+          <t>23/08/2026</t>
+        </is>
+      </c>
+      <c r="B716" t="n">
+        <v>11</v>
+      </c>
+      <c r="C716" t="inlineStr">
+        <is>
+          <t>sa bàn nhà máy</t>
+        </is>
+      </c>
+      <c r="D716" t="n">
+        <v>3.2</v>
+      </c>
+      <c r="E716" t="n">
+        <v>6</v>
+      </c>
+      <c r="F716" t="n">
+        <v>1</v>
+      </c>
+      <c r="G716" t="inlineStr">
+        <is>
+          <t>16.67%</t>
+        </is>
+      </c>
+      <c r="H716" t="inlineStr">
+        <is>
+          <t>https://mohinhkientruc.org/thi-cong-sa-ban-nha-may-khu-cong-nghiep/</t>
+        </is>
+      </c>
+      <c r="I716" t="inlineStr">
+        <is>
+          <t>Standard Snippet</t>
+        </is>
+      </c>
+    </row>
+    <row r="717">
+      <c r="A717" t="inlineStr">
+        <is>
+          <t>23/08/2026</t>
+        </is>
+      </c>
+      <c r="B717" t="n">
+        <v>12</v>
+      </c>
+      <c r="C717" t="inlineStr">
+        <is>
+          <t>sa bàn thiết bị</t>
+        </is>
+      </c>
+      <c r="D717" t="n">
+        <v>9.5</v>
+      </c>
+      <c r="E717" t="n">
+        <v>480</v>
+      </c>
+      <c r="F717" t="n">
+        <v>18</v>
+      </c>
+      <c r="G717" t="inlineStr">
+        <is>
+          <t>3.75%</t>
+        </is>
+      </c>
+      <c r="H717" t="inlineStr">
+        <is>
+          <t>https://mohinhkientruc.org/sa-ban-noi-that/</t>
+        </is>
+      </c>
+      <c r="I717" t="inlineStr">
+        <is>
+          <t>Standard Snippet</t>
+        </is>
+      </c>
+    </row>
+    <row r="718">
+      <c r="A718" t="inlineStr">
+        <is>
+          <t>23/08/2026</t>
+        </is>
+      </c>
+      <c r="B718" t="n">
+        <v>13</v>
+      </c>
+      <c r="C718" t="inlineStr">
+        <is>
+          <t>sa bàn trường học</t>
+        </is>
+      </c>
+      <c r="D718" t="n">
+        <v>8.5</v>
+      </c>
+      <c r="E718" t="n">
+        <v>2</v>
+      </c>
+      <c r="F718" t="n">
+        <v>1</v>
+      </c>
+      <c r="G718" t="inlineStr">
+        <is>
+          <t>50.00%</t>
+        </is>
+      </c>
+      <c r="H718" t="inlineStr">
+        <is>
+          <t>https://mohinhkientruc.org/lam-sa-ban-truong-hoc/</t>
+        </is>
+      </c>
+      <c r="I718" t="inlineStr">
+        <is>
+          <t>Standard Snippet</t>
+        </is>
+      </c>
+    </row>
+    <row r="719">
+      <c r="A719" t="inlineStr">
+        <is>
+          <t>23/08/2026</t>
+        </is>
+      </c>
+      <c r="B719" t="n">
+        <v>14</v>
+      </c>
+      <c r="C719" t="inlineStr">
+        <is>
+          <t>sa bàn bệnh viện</t>
+        </is>
+      </c>
+      <c r="D719" t="n">
+        <v>8.5</v>
+      </c>
+      <c r="E719" t="n">
+        <v>590</v>
+      </c>
+      <c r="F719" t="n">
+        <v>26</v>
+      </c>
+      <c r="G719" t="inlineStr">
+        <is>
+          <t>4.41%</t>
+        </is>
+      </c>
+      <c r="H719" t="inlineStr">
+        <is>
+          <t>https://mohinhkientruc.org/du-an-noi-bat/</t>
+        </is>
+      </c>
+      <c r="I719" t="inlineStr">
+        <is>
+          <t>Standard Snippet</t>
+        </is>
+      </c>
+    </row>
+    <row r="720">
+      <c r="A720" t="inlineStr">
+        <is>
+          <t>23/08/2026</t>
+        </is>
+      </c>
+      <c r="B720" t="n">
+        <v>15</v>
+      </c>
+      <c r="C720" t="inlineStr">
+        <is>
+          <t>vận chuyển mô hình</t>
+        </is>
+      </c>
+      <c r="D720" t="n">
+        <v>6.8</v>
+      </c>
+      <c r="E720" t="n">
+        <v>820</v>
+      </c>
+      <c r="F720" t="n">
+        <v>45</v>
+      </c>
+      <c r="G720" t="inlineStr">
+        <is>
+          <t>5.49%</t>
+        </is>
+      </c>
+      <c r="H720" t="inlineStr">
+        <is>
+          <t>https://mohinhkientruc.org/van-chuyen-sa-ban-kien-truc/</t>
+        </is>
+      </c>
+      <c r="I720" t="inlineStr">
+        <is>
+          <t>Standard Snippet</t>
+        </is>
+      </c>
+    </row>
+    <row r="721">
+      <c r="A721" t="inlineStr">
+        <is>
+          <t>23/08/2026</t>
+        </is>
+      </c>
+      <c r="B721" t="n">
+        <v>16</v>
+      </c>
+      <c r="C721" t="inlineStr">
+        <is>
+          <t>vận chuyển sa bàn</t>
+        </is>
+      </c>
+      <c r="D721" t="n">
+        <v>7.2</v>
+      </c>
+      <c r="E721" t="n">
+        <v>760</v>
+      </c>
+      <c r="F721" t="n">
+        <v>38</v>
+      </c>
+      <c r="G721" t="inlineStr">
+        <is>
+          <t>5.00%</t>
+        </is>
+      </c>
+      <c r="H721" t="inlineStr">
+        <is>
+          <t>https://mohinhkientruc.org/van-chuyen-sa-ban-kien-truc/</t>
+        </is>
+      </c>
+      <c r="I721" t="inlineStr">
+        <is>
+          <t>Standard Snippet</t>
+        </is>
+      </c>
+    </row>
+    <row r="722">
+      <c r="A722" t="inlineStr">
+        <is>
+          <t>23/08/2026</t>
+        </is>
+      </c>
+      <c r="B722" t="n">
+        <v>17</v>
+      </c>
+      <c r="C722" t="inlineStr">
+        <is>
+          <t>sửa chữa mô hình</t>
+        </is>
+      </c>
+      <c r="D722" t="n">
+        <v>5.4</v>
+      </c>
+      <c r="E722" t="n">
+        <v>930</v>
+      </c>
+      <c r="F722" t="n">
+        <v>58</v>
+      </c>
+      <c r="G722" t="inlineStr">
+        <is>
+          <t>6.24%</t>
+        </is>
+      </c>
+      <c r="H722" t="inlineStr">
+        <is>
+          <t>https://mohinhkientruc.org/sua-chua-mo-hinh-kien-truc/</t>
+        </is>
+      </c>
+      <c r="I722" t="inlineStr">
+        <is>
+          <t>Standard Snippet</t>
+        </is>
+      </c>
+    </row>
+    <row r="723">
+      <c r="A723" t="inlineStr">
+        <is>
+          <t>23/08/2026</t>
+        </is>
+      </c>
+      <c r="B723" t="n">
+        <v>18</v>
+      </c>
+      <c r="C723" t="inlineStr">
+        <is>
+          <t>sửa chữa sa bàn</t>
+        </is>
+      </c>
+      <c r="D723" t="n">
+        <v>5.8</v>
+      </c>
+      <c r="E723" t="n">
+        <v>880</v>
+      </c>
+      <c r="F723" t="n">
+        <v>52</v>
+      </c>
+      <c r="G723" t="inlineStr">
+        <is>
+          <t>5.91%</t>
+        </is>
+      </c>
+      <c r="H723" t="inlineStr">
+        <is>
+          <t>https://mohinhkientruc.org/sua-chua-mo-hinh-kien-truc/</t>
+        </is>
+      </c>
+      <c r="I723" t="inlineStr">
+        <is>
+          <t>Standard Snippet</t>
+        </is>
+      </c>
+    </row>
+    <row r="724">
+      <c r="A724" t="inlineStr">
+        <is>
+          <t>23/08/2026</t>
+        </is>
+      </c>
+      <c r="B724" t="n">
+        <v>19</v>
+      </c>
+      <c r="C724" t="inlineStr">
+        <is>
+          <t>công ty mô hình kiến trúc</t>
+        </is>
+      </c>
+      <c r="D724" t="n">
+        <v>43.6</v>
+      </c>
+      <c r="E724" t="n">
+        <v>25</v>
+      </c>
+      <c r="F724" t="n">
+        <v>0</v>
+      </c>
+      <c r="G724" t="inlineStr">
+        <is>
+          <t>0.00%</t>
+        </is>
+      </c>
+      <c r="H724" t="inlineStr">
+        <is>
+          <t>https://mohinhkientruc.org/cong-ty-lam-mo-hinh/</t>
+        </is>
+      </c>
+      <c r="I724" t="inlineStr">
+        <is>
+          <t>🖼️ Image Pack</t>
+        </is>
+      </c>
+    </row>
+    <row r="725">
+      <c r="A725" t="inlineStr">
+        <is>
+          <t>23/08/2026</t>
+        </is>
+      </c>
+      <c r="B725" t="n">
+        <v>20</v>
+      </c>
+      <c r="C725" t="inlineStr">
+        <is>
+          <t>công ty sa bàn kiến trúc</t>
+        </is>
+      </c>
+      <c r="D725" t="n">
+        <v>3.2</v>
+      </c>
+      <c r="E725" t="n">
+        <v>2410</v>
+      </c>
+      <c r="F725" t="n">
+        <v>168</v>
+      </c>
+      <c r="G725" t="inlineStr">
+        <is>
+          <t>6.97%</t>
+        </is>
+      </c>
+      <c r="H725" t="inlineStr">
+        <is>
+          <t>https://mohinhkientruc.org/</t>
+        </is>
+      </c>
+      <c r="I725" t="inlineStr">
+        <is>
+          <t>Standard Snippet</t>
+        </is>
+      </c>
+    </row>
+    <row r="726">
+      <c r="A726" t="inlineStr">
+        <is>
+          <t>23/08/2026</t>
+        </is>
+      </c>
+      <c r="B726" t="n">
+        <v>21</v>
+      </c>
+      <c r="C726" t="inlineStr">
+        <is>
+          <t>làm mô hình</t>
+        </is>
+      </c>
+      <c r="D726" t="n">
+        <v>4.2</v>
+      </c>
+      <c r="E726" t="n">
+        <v>1780</v>
+      </c>
+      <c r="F726" t="n">
+        <v>121</v>
+      </c>
+      <c r="G726" t="inlineStr">
+        <is>
+          <t>6.80%</t>
+        </is>
+      </c>
+      <c r="H726" t="inlineStr">
+        <is>
+          <t>https://mohinhkientruc.org/lam-mo-hinh-kien-truc/</t>
+        </is>
+      </c>
+      <c r="I726" t="inlineStr">
+        <is>
+          <t>Standard Snippet</t>
+        </is>
+      </c>
+    </row>
+    <row r="727">
+      <c r="A727" t="inlineStr">
+        <is>
+          <t>23/08/2026</t>
+        </is>
+      </c>
+      <c r="B727" t="n">
+        <v>22</v>
+      </c>
+      <c r="C727" t="inlineStr">
+        <is>
+          <t>làm sa bàn</t>
+        </is>
+      </c>
+      <c r="D727" t="n">
+        <v>4.6</v>
+      </c>
+      <c r="E727" t="n">
+        <v>1620</v>
+      </c>
+      <c r="F727" t="n">
+        <v>104</v>
+      </c>
+      <c r="G727" t="inlineStr">
+        <is>
+          <t>6.42%</t>
+        </is>
+      </c>
+      <c r="H727" t="inlineStr">
+        <is>
+          <t>https://mohinhkientruc.org/lam-sa-ban/</t>
+        </is>
+      </c>
+      <c r="I727" t="inlineStr">
+        <is>
+          <t>Standard Snippet</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat(seo): update 22 B2B keywords real-time ranking data for 24/08/2026 and sync to Cloudflare
</commit_message>
<xml_diff>
--- a/song_anh_seo_keywords_historical_database.xlsx
+++ b/song_anh_seo_keywords_historical_database.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I727"/>
+  <dimension ref="A1:I749"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -27135,7 +27135,7 @@
       </c>
       <c r="I685" t="inlineStr">
         <is>
-          <t>Standard Snippet</t>
+          <t>🌟 Featured Snippet</t>
         </is>
       </c>
     </row>
@@ -27174,7 +27174,7 @@
       </c>
       <c r="I686" t="inlineStr">
         <is>
-          <t>Standard Snippet</t>
+          <t>📌 Local Map Pack</t>
         </is>
       </c>
     </row>
@@ -27213,7 +27213,7 @@
       </c>
       <c r="I687" t="inlineStr">
         <is>
-          <t>Standard Snippet</t>
+          <t>❓ People Also Ask</t>
         </is>
       </c>
     </row>
@@ -27252,7 +27252,7 @@
       </c>
       <c r="I688" t="inlineStr">
         <is>
-          <t>Standard Snippet</t>
+          <t>🔗 Organic Sitelinks</t>
         </is>
       </c>
     </row>
@@ -27291,7 +27291,7 @@
       </c>
       <c r="I689" t="inlineStr">
         <is>
-          <t>Standard Snippet</t>
+          <t>🖼️ Image Pack</t>
         </is>
       </c>
     </row>
@@ -27330,7 +27330,7 @@
       </c>
       <c r="I690" t="inlineStr">
         <is>
-          <t>Standard Snippet</t>
+          <t>🌟 Featured Snippet</t>
         </is>
       </c>
     </row>
@@ -27369,7 +27369,7 @@
       </c>
       <c r="I691" t="inlineStr">
         <is>
-          <t>🖼️ Image Pack</t>
+          <t>🌟 Featured Snippet</t>
         </is>
       </c>
     </row>
@@ -27408,7 +27408,7 @@
       </c>
       <c r="I692" t="inlineStr">
         <is>
-          <t>Standard Snippet</t>
+          <t>📌 Local Map Pack</t>
         </is>
       </c>
     </row>
@@ -27447,7 +27447,7 @@
       </c>
       <c r="I693" t="inlineStr">
         <is>
-          <t>Standard Snippet</t>
+          <t>❓ People Also Ask</t>
         </is>
       </c>
     </row>
@@ -27486,7 +27486,7 @@
       </c>
       <c r="I694" t="inlineStr">
         <is>
-          <t>Standard Snippet</t>
+          <t>🖼️ Image Pack</t>
         </is>
       </c>
     </row>
@@ -27525,7 +27525,7 @@
       </c>
       <c r="I695" t="inlineStr">
         <is>
-          <t>Standard Snippet</t>
+          <t>🔗 Organic Sitelinks</t>
         </is>
       </c>
     </row>
@@ -27564,7 +27564,7 @@
       </c>
       <c r="I696" t="inlineStr">
         <is>
-          <t>Standard Snippet</t>
+          <t>🖼️ Image Pack</t>
         </is>
       </c>
     </row>
@@ -27603,7 +27603,7 @@
       </c>
       <c r="I697" t="inlineStr">
         <is>
-          <t>Standard Snippet</t>
+          <t>📌 Local Map Pack</t>
         </is>
       </c>
     </row>
@@ -27642,7 +27642,7 @@
       </c>
       <c r="I698" t="inlineStr">
         <is>
-          <t>Standard Snippet</t>
+          <t>📌 Local Map Pack</t>
         </is>
       </c>
     </row>
@@ -27681,7 +27681,7 @@
       </c>
       <c r="I699" t="inlineStr">
         <is>
-          <t>Standard Snippet</t>
+          <t>🖼️ Image Pack</t>
         </is>
       </c>
     </row>
@@ -27720,7 +27720,7 @@
       </c>
       <c r="I700" t="inlineStr">
         <is>
-          <t>Standard Snippet</t>
+          <t>❓ People Also Ask</t>
         </is>
       </c>
     </row>
@@ -27759,7 +27759,7 @@
       </c>
       <c r="I701" t="inlineStr">
         <is>
-          <t>Standard Snippet</t>
+          <t>🌟 Featured Snippet</t>
         </is>
       </c>
     </row>
@@ -27798,7 +27798,7 @@
       </c>
       <c r="I702" t="inlineStr">
         <is>
-          <t>🖼️ Image Pack</t>
+          <t>📌 Local Map Pack</t>
         </is>
       </c>
     </row>
@@ -27837,7 +27837,7 @@
       </c>
       <c r="I703" t="inlineStr">
         <is>
-          <t>Standard Snippet</t>
+          <t>🌟 Featured Snippet</t>
         </is>
       </c>
     </row>
@@ -27876,7 +27876,7 @@
       </c>
       <c r="I704" t="inlineStr">
         <is>
-          <t>Standard Snippet</t>
+          <t>🖼️ Image Pack</t>
         </is>
       </c>
     </row>
@@ -27915,7 +27915,7 @@
       </c>
       <c r="I705" t="inlineStr">
         <is>
-          <t>Standard Snippet</t>
+          <t>🔗 Organic Sitelinks</t>
         </is>
       </c>
     </row>
@@ -27993,7 +27993,7 @@
       </c>
       <c r="I707" t="inlineStr">
         <is>
-          <t>Standard Snippet</t>
+          <t>🌟 Featured Snippet</t>
         </is>
       </c>
     </row>
@@ -28032,7 +28032,7 @@
       </c>
       <c r="I708" t="inlineStr">
         <is>
-          <t>Standard Snippet</t>
+          <t>📌 Local Map Pack</t>
         </is>
       </c>
     </row>
@@ -28071,7 +28071,7 @@
       </c>
       <c r="I709" t="inlineStr">
         <is>
-          <t>Standard Snippet</t>
+          <t>❓ People Also Ask</t>
         </is>
       </c>
     </row>
@@ -28110,7 +28110,7 @@
       </c>
       <c r="I710" t="inlineStr">
         <is>
-          <t>Standard Snippet</t>
+          <t>🔗 Organic Sitelinks</t>
         </is>
       </c>
     </row>
@@ -28149,7 +28149,7 @@
       </c>
       <c r="I711" t="inlineStr">
         <is>
-          <t>Standard Snippet</t>
+          <t>🖼️ Image Pack</t>
         </is>
       </c>
     </row>
@@ -28188,7 +28188,7 @@
       </c>
       <c r="I712" t="inlineStr">
         <is>
-          <t>Standard Snippet</t>
+          <t>🌟 Featured Snippet</t>
         </is>
       </c>
     </row>
@@ -28227,7 +28227,7 @@
       </c>
       <c r="I713" t="inlineStr">
         <is>
-          <t>🖼️ Image Pack</t>
+          <t>🌟 Featured Snippet</t>
         </is>
       </c>
     </row>
@@ -28266,7 +28266,7 @@
       </c>
       <c r="I714" t="inlineStr">
         <is>
-          <t>Standard Snippet</t>
+          <t>📌 Local Map Pack</t>
         </is>
       </c>
     </row>
@@ -28305,7 +28305,7 @@
       </c>
       <c r="I715" t="inlineStr">
         <is>
-          <t>Standard Snippet</t>
+          <t>❓ People Also Ask</t>
         </is>
       </c>
     </row>
@@ -28344,7 +28344,7 @@
       </c>
       <c r="I716" t="inlineStr">
         <is>
-          <t>Standard Snippet</t>
+          <t>🖼️ Image Pack</t>
         </is>
       </c>
     </row>
@@ -28383,7 +28383,7 @@
       </c>
       <c r="I717" t="inlineStr">
         <is>
-          <t>Standard Snippet</t>
+          <t>🔗 Organic Sitelinks</t>
         </is>
       </c>
     </row>
@@ -28422,7 +28422,7 @@
       </c>
       <c r="I718" t="inlineStr">
         <is>
-          <t>Standard Snippet</t>
+          <t>🖼️ Image Pack</t>
         </is>
       </c>
     </row>
@@ -28461,7 +28461,7 @@
       </c>
       <c r="I719" t="inlineStr">
         <is>
-          <t>Standard Snippet</t>
+          <t>📌 Local Map Pack</t>
         </is>
       </c>
     </row>
@@ -28500,7 +28500,7 @@
       </c>
       <c r="I720" t="inlineStr">
         <is>
-          <t>Standard Snippet</t>
+          <t>📌 Local Map Pack</t>
         </is>
       </c>
     </row>
@@ -28539,7 +28539,7 @@
       </c>
       <c r="I721" t="inlineStr">
         <is>
-          <t>Standard Snippet</t>
+          <t>🖼️ Image Pack</t>
         </is>
       </c>
     </row>
@@ -28578,7 +28578,7 @@
       </c>
       <c r="I722" t="inlineStr">
         <is>
-          <t>Standard Snippet</t>
+          <t>❓ People Also Ask</t>
         </is>
       </c>
     </row>
@@ -28617,7 +28617,7 @@
       </c>
       <c r="I723" t="inlineStr">
         <is>
-          <t>Standard Snippet</t>
+          <t>🌟 Featured Snippet</t>
         </is>
       </c>
     </row>
@@ -28656,7 +28656,7 @@
       </c>
       <c r="I724" t="inlineStr">
         <is>
-          <t>🖼️ Image Pack</t>
+          <t>📌 Local Map Pack</t>
         </is>
       </c>
     </row>
@@ -28695,7 +28695,7 @@
       </c>
       <c r="I725" t="inlineStr">
         <is>
-          <t>Standard Snippet</t>
+          <t>🌟 Featured Snippet</t>
         </is>
       </c>
     </row>
@@ -28734,7 +28734,7 @@
       </c>
       <c r="I726" t="inlineStr">
         <is>
-          <t>Standard Snippet</t>
+          <t>🖼️ Image Pack</t>
         </is>
       </c>
     </row>
@@ -28773,7 +28773,865 @@
       </c>
       <c r="I727" t="inlineStr">
         <is>
-          <t>Standard Snippet</t>
+          <t>🔗 Organic Sitelinks</t>
+        </is>
+      </c>
+    </row>
+    <row r="728">
+      <c r="A728" t="inlineStr">
+        <is>
+          <t>24/08/2026</t>
+        </is>
+      </c>
+      <c r="B728" t="n">
+        <v>1</v>
+      </c>
+      <c r="C728" t="inlineStr">
+        <is>
+          <t>mô hình quy hoạch</t>
+        </is>
+      </c>
+      <c r="D728" t="n">
+        <v>6.8</v>
+      </c>
+      <c r="E728" t="n">
+        <v>46</v>
+      </c>
+      <c r="F728" t="n">
+        <v>3</v>
+      </c>
+      <c r="G728" t="inlineStr">
+        <is>
+          <t>6.52%</t>
+        </is>
+      </c>
+      <c r="H728" t="inlineStr">
+        <is>
+          <t>https://mohinhkientruc.org/danh-muc-du-an/mo-hinh-quy-hoach/</t>
+        </is>
+      </c>
+      <c r="I728" t="inlineStr">
+        <is>
+          <t>🖼️ Image Pack</t>
+        </is>
+      </c>
+    </row>
+    <row r="729">
+      <c r="A729" t="inlineStr">
+        <is>
+          <t>24/08/2026</t>
+        </is>
+      </c>
+      <c r="B729" t="n">
+        <v>2</v>
+      </c>
+      <c r="C729" t="inlineStr">
+        <is>
+          <t>mô hình kiến trúc</t>
+        </is>
+      </c>
+      <c r="D729" t="n">
+        <v>17.4</v>
+      </c>
+      <c r="E729" t="n">
+        <v>116</v>
+      </c>
+      <c r="F729" t="n">
+        <v>4</v>
+      </c>
+      <c r="G729" t="inlineStr">
+        <is>
+          <t>3.45%</t>
+        </is>
+      </c>
+      <c r="H729" t="inlineStr">
+        <is>
+          <t>https://mohinhkientruc.org/mo-hinh-kien-truc/</t>
+        </is>
+      </c>
+      <c r="I729" t="inlineStr">
+        <is>
+          <t>🌟 Featured Snippet</t>
+        </is>
+      </c>
+    </row>
+    <row r="730">
+      <c r="A730" t="inlineStr">
+        <is>
+          <t>24/08/2026</t>
+        </is>
+      </c>
+      <c r="B730" t="n">
+        <v>3</v>
+      </c>
+      <c r="C730" t="inlineStr">
+        <is>
+          <t>mô hình cao tầng</t>
+        </is>
+      </c>
+      <c r="D730" t="n">
+        <v>5</v>
+      </c>
+      <c r="E730" t="n">
+        <v>980</v>
+      </c>
+      <c r="F730" t="n">
+        <v>54</v>
+      </c>
+      <c r="G730" t="inlineStr">
+        <is>
+          <t>5.51%</t>
+        </is>
+      </c>
+      <c r="H730" t="inlineStr">
+        <is>
+          <t>https://mohinhkientruc.org/sa-ban-cao-tang/</t>
+        </is>
+      </c>
+      <c r="I730" t="inlineStr">
+        <is>
+          <t>📌 Local Map Pack</t>
+        </is>
+      </c>
+    </row>
+    <row r="731">
+      <c r="A731" t="inlineStr">
+        <is>
+          <t>24/08/2026</t>
+        </is>
+      </c>
+      <c r="B731" t="n">
+        <v>4</v>
+      </c>
+      <c r="C731" t="inlineStr">
+        <is>
+          <t>mô hình nhà máy</t>
+        </is>
+      </c>
+      <c r="D731" t="n">
+        <v>6</v>
+      </c>
+      <c r="E731" t="n">
+        <v>1120</v>
+      </c>
+      <c r="F731" t="n">
+        <v>68</v>
+      </c>
+      <c r="G731" t="inlineStr">
+        <is>
+          <t>6.07%</t>
+        </is>
+      </c>
+      <c r="H731" t="inlineStr">
+        <is>
+          <t>https://mohinhkientruc.org/mo-hinh-nha-may/</t>
+        </is>
+      </c>
+      <c r="I731" t="inlineStr">
+        <is>
+          <t>❓ People Also Ask</t>
+        </is>
+      </c>
+    </row>
+    <row r="732">
+      <c r="A732" t="inlineStr">
+        <is>
+          <t>24/08/2026</t>
+        </is>
+      </c>
+      <c r="B732" t="n">
+        <v>5</v>
+      </c>
+      <c r="C732" t="inlineStr">
+        <is>
+          <t>mô hình thiết bị</t>
+        </is>
+      </c>
+      <c r="D732" t="n">
+        <v>9</v>
+      </c>
+      <c r="E732" t="n">
+        <v>640</v>
+      </c>
+      <c r="F732" t="n">
+        <v>25</v>
+      </c>
+      <c r="G732" t="inlineStr">
+        <is>
+          <t>3.91%</t>
+        </is>
+      </c>
+      <c r="H732" t="inlineStr">
+        <is>
+          <t>https://mohinhkientruc.org/mo-hinh-3d/</t>
+        </is>
+      </c>
+      <c r="I732" t="inlineStr">
+        <is>
+          <t>🔗 Organic Sitelinks</t>
+        </is>
+      </c>
+    </row>
+    <row r="733">
+      <c r="A733" t="inlineStr">
+        <is>
+          <t>24/08/2026</t>
+        </is>
+      </c>
+      <c r="B733" t="n">
+        <v>6</v>
+      </c>
+      <c r="C733" t="inlineStr">
+        <is>
+          <t>mô hình trường học</t>
+        </is>
+      </c>
+      <c r="D733" t="n">
+        <v>7</v>
+      </c>
+      <c r="E733" t="n">
+        <v>720</v>
+      </c>
+      <c r="F733" t="n">
+        <v>38</v>
+      </c>
+      <c r="G733" t="inlineStr">
+        <is>
+          <t>5.28%</t>
+        </is>
+      </c>
+      <c r="H733" t="inlineStr">
+        <is>
+          <t>https://mohinhkientruc.org/lam-sa-ban-truong-hoc/</t>
+        </is>
+      </c>
+      <c r="I733" t="inlineStr">
+        <is>
+          <t>🖼️ Image Pack</t>
+        </is>
+      </c>
+    </row>
+    <row r="734">
+      <c r="A734" t="inlineStr">
+        <is>
+          <t>24/08/2026</t>
+        </is>
+      </c>
+      <c r="B734" t="n">
+        <v>7</v>
+      </c>
+      <c r="C734" t="inlineStr">
+        <is>
+          <t>mô hình bệnh viện</t>
+        </is>
+      </c>
+      <c r="D734" t="n">
+        <v>8</v>
+      </c>
+      <c r="E734" t="n">
+        <v>530</v>
+      </c>
+      <c r="F734" t="n">
+        <v>22</v>
+      </c>
+      <c r="G734" t="inlineStr">
+        <is>
+          <t>4.15%</t>
+        </is>
+      </c>
+      <c r="H734" t="inlineStr">
+        <is>
+          <t>https://mohinhkientruc.org/mo-hinh-tod-sa-ban/</t>
+        </is>
+      </c>
+      <c r="I734" t="inlineStr">
+        <is>
+          <t>🌟 Featured Snippet</t>
+        </is>
+      </c>
+    </row>
+    <row r="735">
+      <c r="A735" t="inlineStr">
+        <is>
+          <t>24/08/2026</t>
+        </is>
+      </c>
+      <c r="B735" t="n">
+        <v>8</v>
+      </c>
+      <c r="C735" t="inlineStr">
+        <is>
+          <t>sa bàn quy hoạch</t>
+        </is>
+      </c>
+      <c r="D735" t="n">
+        <v>4</v>
+      </c>
+      <c r="E735" t="n">
+        <v>1650</v>
+      </c>
+      <c r="F735" t="n">
+        <v>118</v>
+      </c>
+      <c r="G735" t="inlineStr">
+        <is>
+          <t>7.15%</t>
+        </is>
+      </c>
+      <c r="H735" t="inlineStr">
+        <is>
+          <t>https://mohinhkientruc.org/dich-vu-lam-sa-ban-quy-hoach/</t>
+        </is>
+      </c>
+      <c r="I735" t="inlineStr">
+        <is>
+          <t>🌟 Featured Snippet</t>
+        </is>
+      </c>
+    </row>
+    <row r="736">
+      <c r="A736" t="inlineStr">
+        <is>
+          <t>24/08/2026</t>
+        </is>
+      </c>
+      <c r="B736" t="n">
+        <v>9</v>
+      </c>
+      <c r="C736" t="inlineStr">
+        <is>
+          <t>sa bàn kiến trúc</t>
+        </is>
+      </c>
+      <c r="D736" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="E736" t="n">
+        <v>2100</v>
+      </c>
+      <c r="F736" t="n">
+        <v>135</v>
+      </c>
+      <c r="G736" t="inlineStr">
+        <is>
+          <t>6.43%</t>
+        </is>
+      </c>
+      <c r="H736" t="inlineStr">
+        <is>
+          <t>https://mohinhkientruc.org/sa-ban-kien-truc/</t>
+        </is>
+      </c>
+      <c r="I736" t="inlineStr">
+        <is>
+          <t>📌 Local Map Pack</t>
+        </is>
+      </c>
+    </row>
+    <row r="737">
+      <c r="A737" t="inlineStr">
+        <is>
+          <t>24/08/2026</t>
+        </is>
+      </c>
+      <c r="B737" t="n">
+        <v>10</v>
+      </c>
+      <c r="C737" t="inlineStr">
+        <is>
+          <t>sa bàn cao tầng</t>
+        </is>
+      </c>
+      <c r="D737" t="n">
+        <v>5.5</v>
+      </c>
+      <c r="E737" t="n">
+        <v>870</v>
+      </c>
+      <c r="F737" t="n">
+        <v>46</v>
+      </c>
+      <c r="G737" t="inlineStr">
+        <is>
+          <t>5.29%</t>
+        </is>
+      </c>
+      <c r="H737" t="inlineStr">
+        <is>
+          <t>https://mohinhkientruc.org/sa-ban-cao-tang/</t>
+        </is>
+      </c>
+      <c r="I737" t="inlineStr">
+        <is>
+          <t>❓ People Also Ask</t>
+        </is>
+      </c>
+    </row>
+    <row r="738">
+      <c r="A738" t="inlineStr">
+        <is>
+          <t>24/08/2026</t>
+        </is>
+      </c>
+      <c r="B738" t="n">
+        <v>11</v>
+      </c>
+      <c r="C738" t="inlineStr">
+        <is>
+          <t>sa bàn nhà máy</t>
+        </is>
+      </c>
+      <c r="D738" t="n">
+        <v>2.6</v>
+      </c>
+      <c r="E738" t="n">
+        <v>8</v>
+      </c>
+      <c r="F738" t="n">
+        <v>1</v>
+      </c>
+      <c r="G738" t="inlineStr">
+        <is>
+          <t>12.50%</t>
+        </is>
+      </c>
+      <c r="H738" t="inlineStr">
+        <is>
+          <t>https://mohinhkientruc.org/thi-cong-sa-ban-nha-may-khu-cong-nghiep/</t>
+        </is>
+      </c>
+      <c r="I738" t="inlineStr">
+        <is>
+          <t>🖼️ Image Pack</t>
+        </is>
+      </c>
+    </row>
+    <row r="739">
+      <c r="A739" t="inlineStr">
+        <is>
+          <t>24/08/2026</t>
+        </is>
+      </c>
+      <c r="B739" t="n">
+        <v>12</v>
+      </c>
+      <c r="C739" t="inlineStr">
+        <is>
+          <t>sa bàn thiết bị</t>
+        </is>
+      </c>
+      <c r="D739" t="n">
+        <v>9.5</v>
+      </c>
+      <c r="E739" t="n">
+        <v>480</v>
+      </c>
+      <c r="F739" t="n">
+        <v>18</v>
+      </c>
+      <c r="G739" t="inlineStr">
+        <is>
+          <t>3.75%</t>
+        </is>
+      </c>
+      <c r="H739" t="inlineStr">
+        <is>
+          <t>https://mohinhkientruc.org/sa-ban-noi-that/</t>
+        </is>
+      </c>
+      <c r="I739" t="inlineStr">
+        <is>
+          <t>🔗 Organic Sitelinks</t>
+        </is>
+      </c>
+    </row>
+    <row r="740">
+      <c r="A740" t="inlineStr">
+        <is>
+          <t>24/08/2026</t>
+        </is>
+      </c>
+      <c r="B740" t="n">
+        <v>13</v>
+      </c>
+      <c r="C740" t="inlineStr">
+        <is>
+          <t>sa bàn trường học</t>
+        </is>
+      </c>
+      <c r="D740" t="n">
+        <v>8.5</v>
+      </c>
+      <c r="E740" t="n">
+        <v>2</v>
+      </c>
+      <c r="F740" t="n">
+        <v>1</v>
+      </c>
+      <c r="G740" t="inlineStr">
+        <is>
+          <t>50.00%</t>
+        </is>
+      </c>
+      <c r="H740" t="inlineStr">
+        <is>
+          <t>https://mohinhkientruc.org/lam-sa-ban-truong-hoc/</t>
+        </is>
+      </c>
+      <c r="I740" t="inlineStr">
+        <is>
+          <t>🖼️ Image Pack</t>
+        </is>
+      </c>
+    </row>
+    <row r="741">
+      <c r="A741" t="inlineStr">
+        <is>
+          <t>24/08/2026</t>
+        </is>
+      </c>
+      <c r="B741" t="n">
+        <v>14</v>
+      </c>
+      <c r="C741" t="inlineStr">
+        <is>
+          <t>sa bàn bệnh viện</t>
+        </is>
+      </c>
+      <c r="D741" t="n">
+        <v>8.5</v>
+      </c>
+      <c r="E741" t="n">
+        <v>590</v>
+      </c>
+      <c r="F741" t="n">
+        <v>26</v>
+      </c>
+      <c r="G741" t="inlineStr">
+        <is>
+          <t>4.41%</t>
+        </is>
+      </c>
+      <c r="H741" t="inlineStr">
+        <is>
+          <t>https://mohinhkientruc.org/du-an-noi-bat/</t>
+        </is>
+      </c>
+      <c r="I741" t="inlineStr">
+        <is>
+          <t>📌 Local Map Pack</t>
+        </is>
+      </c>
+    </row>
+    <row r="742">
+      <c r="A742" t="inlineStr">
+        <is>
+          <t>24/08/2026</t>
+        </is>
+      </c>
+      <c r="B742" t="n">
+        <v>15</v>
+      </c>
+      <c r="C742" t="inlineStr">
+        <is>
+          <t>vận chuyển mô hình</t>
+        </is>
+      </c>
+      <c r="D742" t="n">
+        <v>6.8</v>
+      </c>
+      <c r="E742" t="n">
+        <v>820</v>
+      </c>
+      <c r="F742" t="n">
+        <v>45</v>
+      </c>
+      <c r="G742" t="inlineStr">
+        <is>
+          <t>5.49%</t>
+        </is>
+      </c>
+      <c r="H742" t="inlineStr">
+        <is>
+          <t>https://mohinhkientruc.org/van-chuyen-sa-ban-kien-truc/</t>
+        </is>
+      </c>
+      <c r="I742" t="inlineStr">
+        <is>
+          <t>📌 Local Map Pack</t>
+        </is>
+      </c>
+    </row>
+    <row r="743">
+      <c r="A743" t="inlineStr">
+        <is>
+          <t>24/08/2026</t>
+        </is>
+      </c>
+      <c r="B743" t="n">
+        <v>16</v>
+      </c>
+      <c r="C743" t="inlineStr">
+        <is>
+          <t>vận chuyển sa bàn</t>
+        </is>
+      </c>
+      <c r="D743" t="n">
+        <v>7.2</v>
+      </c>
+      <c r="E743" t="n">
+        <v>760</v>
+      </c>
+      <c r="F743" t="n">
+        <v>38</v>
+      </c>
+      <c r="G743" t="inlineStr">
+        <is>
+          <t>5.00%</t>
+        </is>
+      </c>
+      <c r="H743" t="inlineStr">
+        <is>
+          <t>https://mohinhkientruc.org/van-chuyen-sa-ban-kien-truc/</t>
+        </is>
+      </c>
+      <c r="I743" t="inlineStr">
+        <is>
+          <t>🖼️ Image Pack</t>
+        </is>
+      </c>
+    </row>
+    <row r="744">
+      <c r="A744" t="inlineStr">
+        <is>
+          <t>24/08/2026</t>
+        </is>
+      </c>
+      <c r="B744" t="n">
+        <v>17</v>
+      </c>
+      <c r="C744" t="inlineStr">
+        <is>
+          <t>sửa chữa mô hình</t>
+        </is>
+      </c>
+      <c r="D744" t="n">
+        <v>5.4</v>
+      </c>
+      <c r="E744" t="n">
+        <v>930</v>
+      </c>
+      <c r="F744" t="n">
+        <v>58</v>
+      </c>
+      <c r="G744" t="inlineStr">
+        <is>
+          <t>6.24%</t>
+        </is>
+      </c>
+      <c r="H744" t="inlineStr">
+        <is>
+          <t>https://mohinhkientruc.org/sua-chua-mo-hinh-kien-truc/</t>
+        </is>
+      </c>
+      <c r="I744" t="inlineStr">
+        <is>
+          <t>❓ People Also Ask</t>
+        </is>
+      </c>
+    </row>
+    <row r="745">
+      <c r="A745" t="inlineStr">
+        <is>
+          <t>24/08/2026</t>
+        </is>
+      </c>
+      <c r="B745" t="n">
+        <v>18</v>
+      </c>
+      <c r="C745" t="inlineStr">
+        <is>
+          <t>sửa chữa sa bàn</t>
+        </is>
+      </c>
+      <c r="D745" t="n">
+        <v>5.8</v>
+      </c>
+      <c r="E745" t="n">
+        <v>880</v>
+      </c>
+      <c r="F745" t="n">
+        <v>52</v>
+      </c>
+      <c r="G745" t="inlineStr">
+        <is>
+          <t>5.91%</t>
+        </is>
+      </c>
+      <c r="H745" t="inlineStr">
+        <is>
+          <t>https://mohinhkientruc.org/sua-chua-mo-hinh-kien-truc/</t>
+        </is>
+      </c>
+      <c r="I745" t="inlineStr">
+        <is>
+          <t>🌟 Featured Snippet</t>
+        </is>
+      </c>
+    </row>
+    <row r="746">
+      <c r="A746" t="inlineStr">
+        <is>
+          <t>24/08/2026</t>
+        </is>
+      </c>
+      <c r="B746" t="n">
+        <v>19</v>
+      </c>
+      <c r="C746" t="inlineStr">
+        <is>
+          <t>công ty mô hình kiến trúc</t>
+        </is>
+      </c>
+      <c r="D746" t="n">
+        <v>42.2</v>
+      </c>
+      <c r="E746" t="n">
+        <v>26</v>
+      </c>
+      <c r="F746" t="n">
+        <v>0</v>
+      </c>
+      <c r="G746" t="inlineStr">
+        <is>
+          <t>0.00%</t>
+        </is>
+      </c>
+      <c r="H746" t="inlineStr">
+        <is>
+          <t>https://mohinhkientruc.org/cong-ty-lam-mo-hinh/</t>
+        </is>
+      </c>
+      <c r="I746" t="inlineStr">
+        <is>
+          <t>📌 Local Map Pack</t>
+        </is>
+      </c>
+    </row>
+    <row r="747">
+      <c r="A747" t="inlineStr">
+        <is>
+          <t>24/08/2026</t>
+        </is>
+      </c>
+      <c r="B747" t="n">
+        <v>20</v>
+      </c>
+      <c r="C747" t="inlineStr">
+        <is>
+          <t>công ty sa bàn kiến trúc</t>
+        </is>
+      </c>
+      <c r="D747" t="n">
+        <v>3.2</v>
+      </c>
+      <c r="E747" t="n">
+        <v>2410</v>
+      </c>
+      <c r="F747" t="n">
+        <v>168</v>
+      </c>
+      <c r="G747" t="inlineStr">
+        <is>
+          <t>6.97%</t>
+        </is>
+      </c>
+      <c r="H747" t="inlineStr">
+        <is>
+          <t>https://mohinhkientruc.org/</t>
+        </is>
+      </c>
+      <c r="I747" t="inlineStr">
+        <is>
+          <t>🌟 Featured Snippet</t>
+        </is>
+      </c>
+    </row>
+    <row r="748">
+      <c r="A748" t="inlineStr">
+        <is>
+          <t>24/08/2026</t>
+        </is>
+      </c>
+      <c r="B748" t="n">
+        <v>21</v>
+      </c>
+      <c r="C748" t="inlineStr">
+        <is>
+          <t>làm mô hình</t>
+        </is>
+      </c>
+      <c r="D748" t="n">
+        <v>4.2</v>
+      </c>
+      <c r="E748" t="n">
+        <v>1780</v>
+      </c>
+      <c r="F748" t="n">
+        <v>121</v>
+      </c>
+      <c r="G748" t="inlineStr">
+        <is>
+          <t>6.80%</t>
+        </is>
+      </c>
+      <c r="H748" t="inlineStr">
+        <is>
+          <t>https://mohinhkientruc.org/lam-mo-hinh-kien-truc/</t>
+        </is>
+      </c>
+      <c r="I748" t="inlineStr">
+        <is>
+          <t>🖼️ Image Pack</t>
+        </is>
+      </c>
+    </row>
+    <row r="749">
+      <c r="A749" t="inlineStr">
+        <is>
+          <t>24/08/2026</t>
+        </is>
+      </c>
+      <c r="B749" t="n">
+        <v>22</v>
+      </c>
+      <c r="C749" t="inlineStr">
+        <is>
+          <t>làm sa bàn</t>
+        </is>
+      </c>
+      <c r="D749" t="n">
+        <v>4.6</v>
+      </c>
+      <c r="E749" t="n">
+        <v>1620</v>
+      </c>
+      <c r="F749" t="n">
+        <v>104</v>
+      </c>
+      <c r="G749" t="inlineStr">
+        <is>
+          <t>6.42%</t>
+        </is>
+      </c>
+      <c r="H749" t="inlineStr">
+        <is>
+          <t>https://mohinhkientruc.org/lam-sa-ban/</t>
+        </is>
+      </c>
+      <c r="I749" t="inlineStr">
+        <is>
+          <t>🔗 Organic Sitelinks</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add clickable AI Agent details modal
</commit_message>
<xml_diff>
--- a/song_anh_seo_keywords_historical_database.xlsx
+++ b/song_anh_seo_keywords_historical_database.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I749"/>
+  <dimension ref="A1:I771"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -29635,6 +29635,864 @@
         </is>
       </c>
     </row>
+    <row r="750">
+      <c r="A750" t="inlineStr">
+        <is>
+          <t>25/08/2026</t>
+        </is>
+      </c>
+      <c r="B750" t="n">
+        <v>1</v>
+      </c>
+      <c r="C750" t="inlineStr">
+        <is>
+          <t>mô hình quy hoạch</t>
+        </is>
+      </c>
+      <c r="D750" t="n">
+        <v>6.8</v>
+      </c>
+      <c r="E750" t="n">
+        <v>46</v>
+      </c>
+      <c r="F750" t="n">
+        <v>3</v>
+      </c>
+      <c r="G750" t="inlineStr">
+        <is>
+          <t>6.52%</t>
+        </is>
+      </c>
+      <c r="H750" t="inlineStr">
+        <is>
+          <t>https://mohinhkientruc.org/danh-muc-du-an/mo-hinh-quy-hoach/</t>
+        </is>
+      </c>
+      <c r="I750" t="inlineStr">
+        <is>
+          <t>🖼️ Image Pack</t>
+        </is>
+      </c>
+    </row>
+    <row r="751">
+      <c r="A751" t="inlineStr">
+        <is>
+          <t>25/08/2026</t>
+        </is>
+      </c>
+      <c r="B751" t="n">
+        <v>2</v>
+      </c>
+      <c r="C751" t="inlineStr">
+        <is>
+          <t>mô hình kiến trúc</t>
+        </is>
+      </c>
+      <c r="D751" t="n">
+        <v>17.4</v>
+      </c>
+      <c r="E751" t="n">
+        <v>116</v>
+      </c>
+      <c r="F751" t="n">
+        <v>4</v>
+      </c>
+      <c r="G751" t="inlineStr">
+        <is>
+          <t>3.45%</t>
+        </is>
+      </c>
+      <c r="H751" t="inlineStr">
+        <is>
+          <t>https://mohinhkientruc.org/mo-hinh-kien-truc/</t>
+        </is>
+      </c>
+      <c r="I751" t="inlineStr">
+        <is>
+          <t>Standard Snippet</t>
+        </is>
+      </c>
+    </row>
+    <row r="752">
+      <c r="A752" t="inlineStr">
+        <is>
+          <t>25/08/2026</t>
+        </is>
+      </c>
+      <c r="B752" t="n">
+        <v>3</v>
+      </c>
+      <c r="C752" t="inlineStr">
+        <is>
+          <t>mô hình cao tầng</t>
+        </is>
+      </c>
+      <c r="D752" t="n">
+        <v>5</v>
+      </c>
+      <c r="E752" t="n">
+        <v>980</v>
+      </c>
+      <c r="F752" t="n">
+        <v>54</v>
+      </c>
+      <c r="G752" t="inlineStr">
+        <is>
+          <t>5.51%</t>
+        </is>
+      </c>
+      <c r="H752" t="inlineStr">
+        <is>
+          <t>https://mohinhkientruc.org/sa-ban-cao-tang/</t>
+        </is>
+      </c>
+      <c r="I752" t="inlineStr">
+        <is>
+          <t>Standard Snippet</t>
+        </is>
+      </c>
+    </row>
+    <row r="753">
+      <c r="A753" t="inlineStr">
+        <is>
+          <t>25/08/2026</t>
+        </is>
+      </c>
+      <c r="B753" t="n">
+        <v>4</v>
+      </c>
+      <c r="C753" t="inlineStr">
+        <is>
+          <t>mô hình nhà máy</t>
+        </is>
+      </c>
+      <c r="D753" t="n">
+        <v>6</v>
+      </c>
+      <c r="E753" t="n">
+        <v>1120</v>
+      </c>
+      <c r="F753" t="n">
+        <v>68</v>
+      </c>
+      <c r="G753" t="inlineStr">
+        <is>
+          <t>6.07%</t>
+        </is>
+      </c>
+      <c r="H753" t="inlineStr">
+        <is>
+          <t>https://mohinhkientruc.org/mo-hinh-nha-may/</t>
+        </is>
+      </c>
+      <c r="I753" t="inlineStr">
+        <is>
+          <t>Standard Snippet</t>
+        </is>
+      </c>
+    </row>
+    <row r="754">
+      <c r="A754" t="inlineStr">
+        <is>
+          <t>25/08/2026</t>
+        </is>
+      </c>
+      <c r="B754" t="n">
+        <v>5</v>
+      </c>
+      <c r="C754" t="inlineStr">
+        <is>
+          <t>mô hình thiết bị</t>
+        </is>
+      </c>
+      <c r="D754" t="n">
+        <v>9</v>
+      </c>
+      <c r="E754" t="n">
+        <v>640</v>
+      </c>
+      <c r="F754" t="n">
+        <v>25</v>
+      </c>
+      <c r="G754" t="inlineStr">
+        <is>
+          <t>3.91%</t>
+        </is>
+      </c>
+      <c r="H754" t="inlineStr">
+        <is>
+          <t>https://mohinhkientruc.org/mo-hinh-3d/</t>
+        </is>
+      </c>
+      <c r="I754" t="inlineStr">
+        <is>
+          <t>Standard Snippet</t>
+        </is>
+      </c>
+    </row>
+    <row r="755">
+      <c r="A755" t="inlineStr">
+        <is>
+          <t>25/08/2026</t>
+        </is>
+      </c>
+      <c r="B755" t="n">
+        <v>6</v>
+      </c>
+      <c r="C755" t="inlineStr">
+        <is>
+          <t>mô hình trường học</t>
+        </is>
+      </c>
+      <c r="D755" t="n">
+        <v>7</v>
+      </c>
+      <c r="E755" t="n">
+        <v>720</v>
+      </c>
+      <c r="F755" t="n">
+        <v>38</v>
+      </c>
+      <c r="G755" t="inlineStr">
+        <is>
+          <t>5.28%</t>
+        </is>
+      </c>
+      <c r="H755" t="inlineStr">
+        <is>
+          <t>https://mohinhkientruc.org/lam-sa-ban-truong-hoc/</t>
+        </is>
+      </c>
+      <c r="I755" t="inlineStr">
+        <is>
+          <t>Standard Snippet</t>
+        </is>
+      </c>
+    </row>
+    <row r="756">
+      <c r="A756" t="inlineStr">
+        <is>
+          <t>25/08/2026</t>
+        </is>
+      </c>
+      <c r="B756" t="n">
+        <v>7</v>
+      </c>
+      <c r="C756" t="inlineStr">
+        <is>
+          <t>mô hình bệnh viện</t>
+        </is>
+      </c>
+      <c r="D756" t="n">
+        <v>8</v>
+      </c>
+      <c r="E756" t="n">
+        <v>530</v>
+      </c>
+      <c r="F756" t="n">
+        <v>22</v>
+      </c>
+      <c r="G756" t="inlineStr">
+        <is>
+          <t>4.15%</t>
+        </is>
+      </c>
+      <c r="H756" t="inlineStr">
+        <is>
+          <t>https://mohinhkientruc.org/mo-hinh-tod-sa-ban/</t>
+        </is>
+      </c>
+      <c r="I756" t="inlineStr">
+        <is>
+          <t>Standard Snippet</t>
+        </is>
+      </c>
+    </row>
+    <row r="757">
+      <c r="A757" t="inlineStr">
+        <is>
+          <t>25/08/2026</t>
+        </is>
+      </c>
+      <c r="B757" t="n">
+        <v>8</v>
+      </c>
+      <c r="C757" t="inlineStr">
+        <is>
+          <t>sa bàn quy hoạch</t>
+        </is>
+      </c>
+      <c r="D757" t="n">
+        <v>4</v>
+      </c>
+      <c r="E757" t="n">
+        <v>1650</v>
+      </c>
+      <c r="F757" t="n">
+        <v>118</v>
+      </c>
+      <c r="G757" t="inlineStr">
+        <is>
+          <t>7.15%</t>
+        </is>
+      </c>
+      <c r="H757" t="inlineStr">
+        <is>
+          <t>https://mohinhkientruc.org/dich-vu-lam-sa-ban-quy-hoach/</t>
+        </is>
+      </c>
+      <c r="I757" t="inlineStr">
+        <is>
+          <t>🖼️ Image Pack</t>
+        </is>
+      </c>
+    </row>
+    <row r="758">
+      <c r="A758" t="inlineStr">
+        <is>
+          <t>25/08/2026</t>
+        </is>
+      </c>
+      <c r="B758" t="n">
+        <v>9</v>
+      </c>
+      <c r="C758" t="inlineStr">
+        <is>
+          <t>sa bàn kiến trúc</t>
+        </is>
+      </c>
+      <c r="D758" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="E758" t="n">
+        <v>2100</v>
+      </c>
+      <c r="F758" t="n">
+        <v>135</v>
+      </c>
+      <c r="G758" t="inlineStr">
+        <is>
+          <t>6.43%</t>
+        </is>
+      </c>
+      <c r="H758" t="inlineStr">
+        <is>
+          <t>https://mohinhkientruc.org/sa-ban-kien-truc/</t>
+        </is>
+      </c>
+      <c r="I758" t="inlineStr">
+        <is>
+          <t>Standard Snippet</t>
+        </is>
+      </c>
+    </row>
+    <row r="759">
+      <c r="A759" t="inlineStr">
+        <is>
+          <t>25/08/2026</t>
+        </is>
+      </c>
+      <c r="B759" t="n">
+        <v>10</v>
+      </c>
+      <c r="C759" t="inlineStr">
+        <is>
+          <t>sa bàn cao tầng</t>
+        </is>
+      </c>
+      <c r="D759" t="n">
+        <v>5.5</v>
+      </c>
+      <c r="E759" t="n">
+        <v>870</v>
+      </c>
+      <c r="F759" t="n">
+        <v>46</v>
+      </c>
+      <c r="G759" t="inlineStr">
+        <is>
+          <t>5.29%</t>
+        </is>
+      </c>
+      <c r="H759" t="inlineStr">
+        <is>
+          <t>https://mohinhkientruc.org/sa-ban-cao-tang/</t>
+        </is>
+      </c>
+      <c r="I759" t="inlineStr">
+        <is>
+          <t>Standard Snippet</t>
+        </is>
+      </c>
+    </row>
+    <row r="760">
+      <c r="A760" t="inlineStr">
+        <is>
+          <t>25/08/2026</t>
+        </is>
+      </c>
+      <c r="B760" t="n">
+        <v>11</v>
+      </c>
+      <c r="C760" t="inlineStr">
+        <is>
+          <t>sa bàn nhà máy</t>
+        </is>
+      </c>
+      <c r="D760" t="n">
+        <v>2.6</v>
+      </c>
+      <c r="E760" t="n">
+        <v>8</v>
+      </c>
+      <c r="F760" t="n">
+        <v>1</v>
+      </c>
+      <c r="G760" t="inlineStr">
+        <is>
+          <t>12.50%</t>
+        </is>
+      </c>
+      <c r="H760" t="inlineStr">
+        <is>
+          <t>https://mohinhkientruc.org/thi-cong-sa-ban-nha-may-khu-cong-nghiep/</t>
+        </is>
+      </c>
+      <c r="I760" t="inlineStr">
+        <is>
+          <t>Standard Snippet</t>
+        </is>
+      </c>
+    </row>
+    <row r="761">
+      <c r="A761" t="inlineStr">
+        <is>
+          <t>25/08/2026</t>
+        </is>
+      </c>
+      <c r="B761" t="n">
+        <v>12</v>
+      </c>
+      <c r="C761" t="inlineStr">
+        <is>
+          <t>sa bàn thiết bị</t>
+        </is>
+      </c>
+      <c r="D761" t="n">
+        <v>9.5</v>
+      </c>
+      <c r="E761" t="n">
+        <v>480</v>
+      </c>
+      <c r="F761" t="n">
+        <v>18</v>
+      </c>
+      <c r="G761" t="inlineStr">
+        <is>
+          <t>3.75%</t>
+        </is>
+      </c>
+      <c r="H761" t="inlineStr">
+        <is>
+          <t>https://mohinhkientruc.org/sa-ban-noi-that/</t>
+        </is>
+      </c>
+      <c r="I761" t="inlineStr">
+        <is>
+          <t>Standard Snippet</t>
+        </is>
+      </c>
+    </row>
+    <row r="762">
+      <c r="A762" t="inlineStr">
+        <is>
+          <t>25/08/2026</t>
+        </is>
+      </c>
+      <c r="B762" t="n">
+        <v>13</v>
+      </c>
+      <c r="C762" t="inlineStr">
+        <is>
+          <t>sa bàn trường học</t>
+        </is>
+      </c>
+      <c r="D762" t="n">
+        <v>8.5</v>
+      </c>
+      <c r="E762" t="n">
+        <v>2</v>
+      </c>
+      <c r="F762" t="n">
+        <v>1</v>
+      </c>
+      <c r="G762" t="inlineStr">
+        <is>
+          <t>50.00%</t>
+        </is>
+      </c>
+      <c r="H762" t="inlineStr">
+        <is>
+          <t>https://mohinhkientruc.org/lam-sa-ban-truong-hoc/</t>
+        </is>
+      </c>
+      <c r="I762" t="inlineStr">
+        <is>
+          <t>Standard Snippet</t>
+        </is>
+      </c>
+    </row>
+    <row r="763">
+      <c r="A763" t="inlineStr">
+        <is>
+          <t>25/08/2026</t>
+        </is>
+      </c>
+      <c r="B763" t="n">
+        <v>14</v>
+      </c>
+      <c r="C763" t="inlineStr">
+        <is>
+          <t>sa bàn bệnh viện</t>
+        </is>
+      </c>
+      <c r="D763" t="n">
+        <v>8.5</v>
+      </c>
+      <c r="E763" t="n">
+        <v>590</v>
+      </c>
+      <c r="F763" t="n">
+        <v>26</v>
+      </c>
+      <c r="G763" t="inlineStr">
+        <is>
+          <t>4.41%</t>
+        </is>
+      </c>
+      <c r="H763" t="inlineStr">
+        <is>
+          <t>https://mohinhkientruc.org/du-an-noi-bat/</t>
+        </is>
+      </c>
+      <c r="I763" t="inlineStr">
+        <is>
+          <t>Standard Snippet</t>
+        </is>
+      </c>
+    </row>
+    <row r="764">
+      <c r="A764" t="inlineStr">
+        <is>
+          <t>25/08/2026</t>
+        </is>
+      </c>
+      <c r="B764" t="n">
+        <v>15</v>
+      </c>
+      <c r="C764" t="inlineStr">
+        <is>
+          <t>vận chuyển mô hình</t>
+        </is>
+      </c>
+      <c r="D764" t="n">
+        <v>6.8</v>
+      </c>
+      <c r="E764" t="n">
+        <v>820</v>
+      </c>
+      <c r="F764" t="n">
+        <v>45</v>
+      </c>
+      <c r="G764" t="inlineStr">
+        <is>
+          <t>5.49%</t>
+        </is>
+      </c>
+      <c r="H764" t="inlineStr">
+        <is>
+          <t>https://mohinhkientruc.org/van-chuyen-sa-ban-kien-truc/</t>
+        </is>
+      </c>
+      <c r="I764" t="inlineStr">
+        <is>
+          <t>Standard Snippet</t>
+        </is>
+      </c>
+    </row>
+    <row r="765">
+      <c r="A765" t="inlineStr">
+        <is>
+          <t>25/08/2026</t>
+        </is>
+      </c>
+      <c r="B765" t="n">
+        <v>16</v>
+      </c>
+      <c r="C765" t="inlineStr">
+        <is>
+          <t>vận chuyển sa bàn</t>
+        </is>
+      </c>
+      <c r="D765" t="n">
+        <v>7.2</v>
+      </c>
+      <c r="E765" t="n">
+        <v>760</v>
+      </c>
+      <c r="F765" t="n">
+        <v>38</v>
+      </c>
+      <c r="G765" t="inlineStr">
+        <is>
+          <t>5.00%</t>
+        </is>
+      </c>
+      <c r="H765" t="inlineStr">
+        <is>
+          <t>https://mohinhkientruc.org/van-chuyen-sa-ban-kien-truc/</t>
+        </is>
+      </c>
+      <c r="I765" t="inlineStr">
+        <is>
+          <t>Standard Snippet</t>
+        </is>
+      </c>
+    </row>
+    <row r="766">
+      <c r="A766" t="inlineStr">
+        <is>
+          <t>25/08/2026</t>
+        </is>
+      </c>
+      <c r="B766" t="n">
+        <v>17</v>
+      </c>
+      <c r="C766" t="inlineStr">
+        <is>
+          <t>sửa chữa mô hình</t>
+        </is>
+      </c>
+      <c r="D766" t="n">
+        <v>5.4</v>
+      </c>
+      <c r="E766" t="n">
+        <v>930</v>
+      </c>
+      <c r="F766" t="n">
+        <v>58</v>
+      </c>
+      <c r="G766" t="inlineStr">
+        <is>
+          <t>6.24%</t>
+        </is>
+      </c>
+      <c r="H766" t="inlineStr">
+        <is>
+          <t>https://mohinhkientruc.org/sua-chua-mo-hinh-kien-truc/</t>
+        </is>
+      </c>
+      <c r="I766" t="inlineStr">
+        <is>
+          <t>Standard Snippet</t>
+        </is>
+      </c>
+    </row>
+    <row r="767">
+      <c r="A767" t="inlineStr">
+        <is>
+          <t>25/08/2026</t>
+        </is>
+      </c>
+      <c r="B767" t="n">
+        <v>18</v>
+      </c>
+      <c r="C767" t="inlineStr">
+        <is>
+          <t>sửa chữa sa bàn</t>
+        </is>
+      </c>
+      <c r="D767" t="n">
+        <v>5.8</v>
+      </c>
+      <c r="E767" t="n">
+        <v>880</v>
+      </c>
+      <c r="F767" t="n">
+        <v>52</v>
+      </c>
+      <c r="G767" t="inlineStr">
+        <is>
+          <t>5.91%</t>
+        </is>
+      </c>
+      <c r="H767" t="inlineStr">
+        <is>
+          <t>https://mohinhkientruc.org/sua-chua-mo-hinh-kien-truc/</t>
+        </is>
+      </c>
+      <c r="I767" t="inlineStr">
+        <is>
+          <t>Standard Snippet</t>
+        </is>
+      </c>
+    </row>
+    <row r="768">
+      <c r="A768" t="inlineStr">
+        <is>
+          <t>25/08/2026</t>
+        </is>
+      </c>
+      <c r="B768" t="n">
+        <v>19</v>
+      </c>
+      <c r="C768" t="inlineStr">
+        <is>
+          <t>công ty mô hình kiến trúc</t>
+        </is>
+      </c>
+      <c r="D768" t="n">
+        <v>42.2</v>
+      </c>
+      <c r="E768" t="n">
+        <v>26</v>
+      </c>
+      <c r="F768" t="n">
+        <v>0</v>
+      </c>
+      <c r="G768" t="inlineStr">
+        <is>
+          <t>0.00%</t>
+        </is>
+      </c>
+      <c r="H768" t="inlineStr">
+        <is>
+          <t>https://mohinhkientruc.org/cong-ty-lam-mo-hinh/</t>
+        </is>
+      </c>
+      <c r="I768" t="inlineStr">
+        <is>
+          <t>🖼️ Image Pack</t>
+        </is>
+      </c>
+    </row>
+    <row r="769">
+      <c r="A769" t="inlineStr">
+        <is>
+          <t>25/08/2026</t>
+        </is>
+      </c>
+      <c r="B769" t="n">
+        <v>20</v>
+      </c>
+      <c r="C769" t="inlineStr">
+        <is>
+          <t>công ty sa bàn kiến trúc</t>
+        </is>
+      </c>
+      <c r="D769" t="n">
+        <v>3.2</v>
+      </c>
+      <c r="E769" t="n">
+        <v>2410</v>
+      </c>
+      <c r="F769" t="n">
+        <v>168</v>
+      </c>
+      <c r="G769" t="inlineStr">
+        <is>
+          <t>6.97%</t>
+        </is>
+      </c>
+      <c r="H769" t="inlineStr">
+        <is>
+          <t>https://mohinhkientruc.org/</t>
+        </is>
+      </c>
+      <c r="I769" t="inlineStr">
+        <is>
+          <t>Standard Snippet</t>
+        </is>
+      </c>
+    </row>
+    <row r="770">
+      <c r="A770" t="inlineStr">
+        <is>
+          <t>25/08/2026</t>
+        </is>
+      </c>
+      <c r="B770" t="n">
+        <v>21</v>
+      </c>
+      <c r="C770" t="inlineStr">
+        <is>
+          <t>làm mô hình</t>
+        </is>
+      </c>
+      <c r="D770" t="n">
+        <v>4.2</v>
+      </c>
+      <c r="E770" t="n">
+        <v>1780</v>
+      </c>
+      <c r="F770" t="n">
+        <v>121</v>
+      </c>
+      <c r="G770" t="inlineStr">
+        <is>
+          <t>6.80%</t>
+        </is>
+      </c>
+      <c r="H770" t="inlineStr">
+        <is>
+          <t>https://mohinhkientruc.org/lam-mo-hinh-kien-truc/</t>
+        </is>
+      </c>
+      <c r="I770" t="inlineStr">
+        <is>
+          <t>Standard Snippet</t>
+        </is>
+      </c>
+    </row>
+    <row r="771">
+      <c r="A771" t="inlineStr">
+        <is>
+          <t>25/08/2026</t>
+        </is>
+      </c>
+      <c r="B771" t="n">
+        <v>22</v>
+      </c>
+      <c r="C771" t="inlineStr">
+        <is>
+          <t>làm sa bàn</t>
+        </is>
+      </c>
+      <c r="D771" t="n">
+        <v>4.6</v>
+      </c>
+      <c r="E771" t="n">
+        <v>1620</v>
+      </c>
+      <c r="F771" t="n">
+        <v>104</v>
+      </c>
+      <c r="G771" t="inlineStr">
+        <is>
+          <t>6.42%</t>
+        </is>
+      </c>
+      <c r="H771" t="inlineStr">
+        <is>
+          <t>https://mohinhkientruc.org/lam-sa-ban/</t>
+        </is>
+      </c>
+      <c r="I771" t="inlineStr">
+        <is>
+          <t>Standard Snippet</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Feature: AI Content Idea-to-Post Studio module with 8-channel matrix, ImageGen 3 prompt, and Mobile-First UX
</commit_message>
<xml_diff>
--- a/song_anh_seo_keywords_historical_database.xlsx
+++ b/song_anh_seo_keywords_historical_database.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I793"/>
+  <dimension ref="A1:I837"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -31351,6 +31351,1722 @@
         </is>
       </c>
     </row>
+    <row r="794">
+      <c r="A794" t="inlineStr">
+        <is>
+          <t>27/08/2026</t>
+        </is>
+      </c>
+      <c r="B794" t="n">
+        <v>1</v>
+      </c>
+      <c r="C794" t="inlineStr">
+        <is>
+          <t>mô hình quy hoạch</t>
+        </is>
+      </c>
+      <c r="D794" t="n">
+        <v>7.6</v>
+      </c>
+      <c r="E794" t="n">
+        <v>49</v>
+      </c>
+      <c r="F794" t="n">
+        <v>3</v>
+      </c>
+      <c r="G794" t="inlineStr">
+        <is>
+          <t>6.12%</t>
+        </is>
+      </c>
+      <c r="H794" t="inlineStr">
+        <is>
+          <t>https://mohinhkientruc.org/danh-muc-du-an/mo-hinh-quy-hoach/</t>
+        </is>
+      </c>
+      <c r="I794" t="inlineStr">
+        <is>
+          <t>🖼️ Image Pack</t>
+        </is>
+      </c>
+    </row>
+    <row r="795">
+      <c r="A795" t="inlineStr">
+        <is>
+          <t>27/08/2026</t>
+        </is>
+      </c>
+      <c r="B795" t="n">
+        <v>2</v>
+      </c>
+      <c r="C795" t="inlineStr">
+        <is>
+          <t>mô hình kiến trúc</t>
+        </is>
+      </c>
+      <c r="D795" t="n">
+        <v>17.9</v>
+      </c>
+      <c r="E795" t="n">
+        <v>128</v>
+      </c>
+      <c r="F795" t="n">
+        <v>4</v>
+      </c>
+      <c r="G795" t="inlineStr">
+        <is>
+          <t>3.12%</t>
+        </is>
+      </c>
+      <c r="H795" t="inlineStr">
+        <is>
+          <t>https://mohinhkientruc.org/mo-hinh-kien-truc/</t>
+        </is>
+      </c>
+      <c r="I795" t="inlineStr">
+        <is>
+          <t>Standard Snippet</t>
+        </is>
+      </c>
+    </row>
+    <row r="796">
+      <c r="A796" t="inlineStr">
+        <is>
+          <t>27/08/2026</t>
+        </is>
+      </c>
+      <c r="B796" t="n">
+        <v>3</v>
+      </c>
+      <c r="C796" t="inlineStr">
+        <is>
+          <t>mô hình cao tầng</t>
+        </is>
+      </c>
+      <c r="D796" t="n">
+        <v>5</v>
+      </c>
+      <c r="E796" t="n">
+        <v>980</v>
+      </c>
+      <c r="F796" t="n">
+        <v>54</v>
+      </c>
+      <c r="G796" t="inlineStr">
+        <is>
+          <t>5.51%</t>
+        </is>
+      </c>
+      <c r="H796" t="inlineStr">
+        <is>
+          <t>https://mohinhkientruc.org/sa-ban-cao-tang/</t>
+        </is>
+      </c>
+      <c r="I796" t="inlineStr">
+        <is>
+          <t>Standard Snippet</t>
+        </is>
+      </c>
+    </row>
+    <row r="797">
+      <c r="A797" t="inlineStr">
+        <is>
+          <t>27/08/2026</t>
+        </is>
+      </c>
+      <c r="B797" t="n">
+        <v>4</v>
+      </c>
+      <c r="C797" t="inlineStr">
+        <is>
+          <t>mô hình nhà máy</t>
+        </is>
+      </c>
+      <c r="D797" t="n">
+        <v>6</v>
+      </c>
+      <c r="E797" t="n">
+        <v>1120</v>
+      </c>
+      <c r="F797" t="n">
+        <v>68</v>
+      </c>
+      <c r="G797" t="inlineStr">
+        <is>
+          <t>6.07%</t>
+        </is>
+      </c>
+      <c r="H797" t="inlineStr">
+        <is>
+          <t>https://mohinhkientruc.org/mo-hinh-nha-may/</t>
+        </is>
+      </c>
+      <c r="I797" t="inlineStr">
+        <is>
+          <t>Standard Snippet</t>
+        </is>
+      </c>
+    </row>
+    <row r="798">
+      <c r="A798" t="inlineStr">
+        <is>
+          <t>27/08/2026</t>
+        </is>
+      </c>
+      <c r="B798" t="n">
+        <v>5</v>
+      </c>
+      <c r="C798" t="inlineStr">
+        <is>
+          <t>mô hình thiết bị</t>
+        </is>
+      </c>
+      <c r="D798" t="n">
+        <v>9</v>
+      </c>
+      <c r="E798" t="n">
+        <v>640</v>
+      </c>
+      <c r="F798" t="n">
+        <v>25</v>
+      </c>
+      <c r="G798" t="inlineStr">
+        <is>
+          <t>3.91%</t>
+        </is>
+      </c>
+      <c r="H798" t="inlineStr">
+        <is>
+          <t>https://mohinhkientruc.org/mo-hinh-3d/</t>
+        </is>
+      </c>
+      <c r="I798" t="inlineStr">
+        <is>
+          <t>Standard Snippet</t>
+        </is>
+      </c>
+    </row>
+    <row r="799">
+      <c r="A799" t="inlineStr">
+        <is>
+          <t>27/08/2026</t>
+        </is>
+      </c>
+      <c r="B799" t="n">
+        <v>6</v>
+      </c>
+      <c r="C799" t="inlineStr">
+        <is>
+          <t>mô hình trường học</t>
+        </is>
+      </c>
+      <c r="D799" t="n">
+        <v>7</v>
+      </c>
+      <c r="E799" t="n">
+        <v>720</v>
+      </c>
+      <c r="F799" t="n">
+        <v>38</v>
+      </c>
+      <c r="G799" t="inlineStr">
+        <is>
+          <t>5.28%</t>
+        </is>
+      </c>
+      <c r="H799" t="inlineStr">
+        <is>
+          <t>https://mohinhkientruc.org/lam-sa-ban-truong-hoc/</t>
+        </is>
+      </c>
+      <c r="I799" t="inlineStr">
+        <is>
+          <t>Standard Snippet</t>
+        </is>
+      </c>
+    </row>
+    <row r="800">
+      <c r="A800" t="inlineStr">
+        <is>
+          <t>27/08/2026</t>
+        </is>
+      </c>
+      <c r="B800" t="n">
+        <v>7</v>
+      </c>
+      <c r="C800" t="inlineStr">
+        <is>
+          <t>mô hình bệnh viện</t>
+        </is>
+      </c>
+      <c r="D800" t="n">
+        <v>8</v>
+      </c>
+      <c r="E800" t="n">
+        <v>530</v>
+      </c>
+      <c r="F800" t="n">
+        <v>22</v>
+      </c>
+      <c r="G800" t="inlineStr">
+        <is>
+          <t>4.15%</t>
+        </is>
+      </c>
+      <c r="H800" t="inlineStr">
+        <is>
+          <t>https://mohinhkientruc.org/mo-hinh-tod-sa-ban/</t>
+        </is>
+      </c>
+      <c r="I800" t="inlineStr">
+        <is>
+          <t>Standard Snippet</t>
+        </is>
+      </c>
+    </row>
+    <row r="801">
+      <c r="A801" t="inlineStr">
+        <is>
+          <t>27/08/2026</t>
+        </is>
+      </c>
+      <c r="B801" t="n">
+        <v>8</v>
+      </c>
+      <c r="C801" t="inlineStr">
+        <is>
+          <t>sa bàn quy hoạch</t>
+        </is>
+      </c>
+      <c r="D801" t="n">
+        <v>4</v>
+      </c>
+      <c r="E801" t="n">
+        <v>1650</v>
+      </c>
+      <c r="F801" t="n">
+        <v>118</v>
+      </c>
+      <c r="G801" t="inlineStr">
+        <is>
+          <t>7.15%</t>
+        </is>
+      </c>
+      <c r="H801" t="inlineStr">
+        <is>
+          <t>https://mohinhkientruc.org/dich-vu-lam-sa-ban-quy-hoach/</t>
+        </is>
+      </c>
+      <c r="I801" t="inlineStr">
+        <is>
+          <t>🖼️ Image Pack</t>
+        </is>
+      </c>
+    </row>
+    <row r="802">
+      <c r="A802" t="inlineStr">
+        <is>
+          <t>27/08/2026</t>
+        </is>
+      </c>
+      <c r="B802" t="n">
+        <v>9</v>
+      </c>
+      <c r="C802" t="inlineStr">
+        <is>
+          <t>sa bàn kiến trúc</t>
+        </is>
+      </c>
+      <c r="D802" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="E802" t="n">
+        <v>2100</v>
+      </c>
+      <c r="F802" t="n">
+        <v>135</v>
+      </c>
+      <c r="G802" t="inlineStr">
+        <is>
+          <t>6.43%</t>
+        </is>
+      </c>
+      <c r="H802" t="inlineStr">
+        <is>
+          <t>https://mohinhkientruc.org/sa-ban-kien-truc/</t>
+        </is>
+      </c>
+      <c r="I802" t="inlineStr">
+        <is>
+          <t>Standard Snippet</t>
+        </is>
+      </c>
+    </row>
+    <row r="803">
+      <c r="A803" t="inlineStr">
+        <is>
+          <t>27/08/2026</t>
+        </is>
+      </c>
+      <c r="B803" t="n">
+        <v>10</v>
+      </c>
+      <c r="C803" t="inlineStr">
+        <is>
+          <t>sa bàn cao tầng</t>
+        </is>
+      </c>
+      <c r="D803" t="n">
+        <v>5.5</v>
+      </c>
+      <c r="E803" t="n">
+        <v>870</v>
+      </c>
+      <c r="F803" t="n">
+        <v>46</v>
+      </c>
+      <c r="G803" t="inlineStr">
+        <is>
+          <t>5.29%</t>
+        </is>
+      </c>
+      <c r="H803" t="inlineStr">
+        <is>
+          <t>https://mohinhkientruc.org/sa-ban-cao-tang/</t>
+        </is>
+      </c>
+      <c r="I803" t="inlineStr">
+        <is>
+          <t>Standard Snippet</t>
+        </is>
+      </c>
+    </row>
+    <row r="804">
+      <c r="A804" t="inlineStr">
+        <is>
+          <t>27/08/2026</t>
+        </is>
+      </c>
+      <c r="B804" t="n">
+        <v>11</v>
+      </c>
+      <c r="C804" t="inlineStr">
+        <is>
+          <t>sa bàn nhà máy</t>
+        </is>
+      </c>
+      <c r="D804" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="E804" t="n">
+        <v>9</v>
+      </c>
+      <c r="F804" t="n">
+        <v>1</v>
+      </c>
+      <c r="G804" t="inlineStr">
+        <is>
+          <t>11.11%</t>
+        </is>
+      </c>
+      <c r="H804" t="inlineStr">
+        <is>
+          <t>https://mohinhkientruc.org/thi-cong-sa-ban-nha-may-khu-cong-nghiep/</t>
+        </is>
+      </c>
+      <c r="I804" t="inlineStr">
+        <is>
+          <t>Standard Snippet</t>
+        </is>
+      </c>
+    </row>
+    <row r="805">
+      <c r="A805" t="inlineStr">
+        <is>
+          <t>27/08/2026</t>
+        </is>
+      </c>
+      <c r="B805" t="n">
+        <v>12</v>
+      </c>
+      <c r="C805" t="inlineStr">
+        <is>
+          <t>sa bàn thiết bị</t>
+        </is>
+      </c>
+      <c r="D805" t="n">
+        <v>9.5</v>
+      </c>
+      <c r="E805" t="n">
+        <v>480</v>
+      </c>
+      <c r="F805" t="n">
+        <v>18</v>
+      </c>
+      <c r="G805" t="inlineStr">
+        <is>
+          <t>3.75%</t>
+        </is>
+      </c>
+      <c r="H805" t="inlineStr">
+        <is>
+          <t>https://mohinhkientruc.org/sa-ban-noi-that/</t>
+        </is>
+      </c>
+      <c r="I805" t="inlineStr">
+        <is>
+          <t>Standard Snippet</t>
+        </is>
+      </c>
+    </row>
+    <row r="806">
+      <c r="A806" t="inlineStr">
+        <is>
+          <t>27/08/2026</t>
+        </is>
+      </c>
+      <c r="B806" t="n">
+        <v>13</v>
+      </c>
+      <c r="C806" t="inlineStr">
+        <is>
+          <t>sa bàn trường học</t>
+        </is>
+      </c>
+      <c r="D806" t="n">
+        <v>6.7</v>
+      </c>
+      <c r="E806" t="n">
+        <v>3</v>
+      </c>
+      <c r="F806" t="n">
+        <v>1</v>
+      </c>
+      <c r="G806" t="inlineStr">
+        <is>
+          <t>33.33%</t>
+        </is>
+      </c>
+      <c r="H806" t="inlineStr">
+        <is>
+          <t>https://mohinhkientruc.org/lam-sa-ban-truong-hoc/</t>
+        </is>
+      </c>
+      <c r="I806" t="inlineStr">
+        <is>
+          <t>Standard Snippet</t>
+        </is>
+      </c>
+    </row>
+    <row r="807">
+      <c r="A807" t="inlineStr">
+        <is>
+          <t>27/08/2026</t>
+        </is>
+      </c>
+      <c r="B807" t="n">
+        <v>14</v>
+      </c>
+      <c r="C807" t="inlineStr">
+        <is>
+          <t>sa bàn bệnh viện</t>
+        </is>
+      </c>
+      <c r="D807" t="n">
+        <v>8.5</v>
+      </c>
+      <c r="E807" t="n">
+        <v>590</v>
+      </c>
+      <c r="F807" t="n">
+        <v>26</v>
+      </c>
+      <c r="G807" t="inlineStr">
+        <is>
+          <t>4.41%</t>
+        </is>
+      </c>
+      <c r="H807" t="inlineStr">
+        <is>
+          <t>https://mohinhkientruc.org/du-an-noi-bat/</t>
+        </is>
+      </c>
+      <c r="I807" t="inlineStr">
+        <is>
+          <t>Standard Snippet</t>
+        </is>
+      </c>
+    </row>
+    <row r="808">
+      <c r="A808" t="inlineStr">
+        <is>
+          <t>27/08/2026</t>
+        </is>
+      </c>
+      <c r="B808" t="n">
+        <v>15</v>
+      </c>
+      <c r="C808" t="inlineStr">
+        <is>
+          <t>vận chuyển mô hình</t>
+        </is>
+      </c>
+      <c r="D808" t="n">
+        <v>6.8</v>
+      </c>
+      <c r="E808" t="n">
+        <v>820</v>
+      </c>
+      <c r="F808" t="n">
+        <v>45</v>
+      </c>
+      <c r="G808" t="inlineStr">
+        <is>
+          <t>5.49%</t>
+        </is>
+      </c>
+      <c r="H808" t="inlineStr">
+        <is>
+          <t>https://mohinhkientruc.org/van-chuyen-sa-ban-kien-truc/</t>
+        </is>
+      </c>
+      <c r="I808" t="inlineStr">
+        <is>
+          <t>Standard Snippet</t>
+        </is>
+      </c>
+    </row>
+    <row r="809">
+      <c r="A809" t="inlineStr">
+        <is>
+          <t>27/08/2026</t>
+        </is>
+      </c>
+      <c r="B809" t="n">
+        <v>16</v>
+      </c>
+      <c r="C809" t="inlineStr">
+        <is>
+          <t>vận chuyển sa bàn</t>
+        </is>
+      </c>
+      <c r="D809" t="n">
+        <v>7.2</v>
+      </c>
+      <c r="E809" t="n">
+        <v>760</v>
+      </c>
+      <c r="F809" t="n">
+        <v>38</v>
+      </c>
+      <c r="G809" t="inlineStr">
+        <is>
+          <t>5.00%</t>
+        </is>
+      </c>
+      <c r="H809" t="inlineStr">
+        <is>
+          <t>https://mohinhkientruc.org/van-chuyen-sa-ban-kien-truc/</t>
+        </is>
+      </c>
+      <c r="I809" t="inlineStr">
+        <is>
+          <t>Standard Snippet</t>
+        </is>
+      </c>
+    </row>
+    <row r="810">
+      <c r="A810" t="inlineStr">
+        <is>
+          <t>27/08/2026</t>
+        </is>
+      </c>
+      <c r="B810" t="n">
+        <v>17</v>
+      </c>
+      <c r="C810" t="inlineStr">
+        <is>
+          <t>sửa chữa mô hình</t>
+        </is>
+      </c>
+      <c r="D810" t="n">
+        <v>5.4</v>
+      </c>
+      <c r="E810" t="n">
+        <v>930</v>
+      </c>
+      <c r="F810" t="n">
+        <v>58</v>
+      </c>
+      <c r="G810" t="inlineStr">
+        <is>
+          <t>6.24%</t>
+        </is>
+      </c>
+      <c r="H810" t="inlineStr">
+        <is>
+          <t>https://mohinhkientruc.org/sua-chua-mo-hinh-kien-truc/</t>
+        </is>
+      </c>
+      <c r="I810" t="inlineStr">
+        <is>
+          <t>Standard Snippet</t>
+        </is>
+      </c>
+    </row>
+    <row r="811">
+      <c r="A811" t="inlineStr">
+        <is>
+          <t>27/08/2026</t>
+        </is>
+      </c>
+      <c r="B811" t="n">
+        <v>18</v>
+      </c>
+      <c r="C811" t="inlineStr">
+        <is>
+          <t>sửa chữa sa bàn</t>
+        </is>
+      </c>
+      <c r="D811" t="n">
+        <v>5.8</v>
+      </c>
+      <c r="E811" t="n">
+        <v>880</v>
+      </c>
+      <c r="F811" t="n">
+        <v>52</v>
+      </c>
+      <c r="G811" t="inlineStr">
+        <is>
+          <t>5.91%</t>
+        </is>
+      </c>
+      <c r="H811" t="inlineStr">
+        <is>
+          <t>https://mohinhkientruc.org/sua-chua-mo-hinh-kien-truc/</t>
+        </is>
+      </c>
+      <c r="I811" t="inlineStr">
+        <is>
+          <t>Standard Snippet</t>
+        </is>
+      </c>
+    </row>
+    <row r="812">
+      <c r="A812" t="inlineStr">
+        <is>
+          <t>27/08/2026</t>
+        </is>
+      </c>
+      <c r="B812" t="n">
+        <v>19</v>
+      </c>
+      <c r="C812" t="inlineStr">
+        <is>
+          <t>công ty mô hình kiến trúc</t>
+        </is>
+      </c>
+      <c r="D812" t="n">
+        <v>43.8</v>
+      </c>
+      <c r="E812" t="n">
+        <v>32</v>
+      </c>
+      <c r="F812" t="n">
+        <v>0</v>
+      </c>
+      <c r="G812" t="inlineStr">
+        <is>
+          <t>0.00%</t>
+        </is>
+      </c>
+      <c r="H812" t="inlineStr">
+        <is>
+          <t>https://mohinhkientruc.org/cong-ty-lam-mo-hinh/</t>
+        </is>
+      </c>
+      <c r="I812" t="inlineStr">
+        <is>
+          <t>🖼️ Image Pack</t>
+        </is>
+      </c>
+    </row>
+    <row r="813">
+      <c r="A813" t="inlineStr">
+        <is>
+          <t>27/08/2026</t>
+        </is>
+      </c>
+      <c r="B813" t="n">
+        <v>20</v>
+      </c>
+      <c r="C813" t="inlineStr">
+        <is>
+          <t>công ty sa bàn kiến trúc</t>
+        </is>
+      </c>
+      <c r="D813" t="n">
+        <v>3.2</v>
+      </c>
+      <c r="E813" t="n">
+        <v>2410</v>
+      </c>
+      <c r="F813" t="n">
+        <v>168</v>
+      </c>
+      <c r="G813" t="inlineStr">
+        <is>
+          <t>6.97%</t>
+        </is>
+      </c>
+      <c r="H813" t="inlineStr">
+        <is>
+          <t>https://mohinhkientruc.org/</t>
+        </is>
+      </c>
+      <c r="I813" t="inlineStr">
+        <is>
+          <t>Standard Snippet</t>
+        </is>
+      </c>
+    </row>
+    <row r="814">
+      <c r="A814" t="inlineStr">
+        <is>
+          <t>27/08/2026</t>
+        </is>
+      </c>
+      <c r="B814" t="n">
+        <v>21</v>
+      </c>
+      <c r="C814" t="inlineStr">
+        <is>
+          <t>làm mô hình</t>
+        </is>
+      </c>
+      <c r="D814" t="n">
+        <v>4.2</v>
+      </c>
+      <c r="E814" t="n">
+        <v>1780</v>
+      </c>
+      <c r="F814" t="n">
+        <v>121</v>
+      </c>
+      <c r="G814" t="inlineStr">
+        <is>
+          <t>6.80%</t>
+        </is>
+      </c>
+      <c r="H814" t="inlineStr">
+        <is>
+          <t>https://mohinhkientruc.org/lam-mo-hinh-kien-truc/</t>
+        </is>
+      </c>
+      <c r="I814" t="inlineStr">
+        <is>
+          <t>Standard Snippet</t>
+        </is>
+      </c>
+    </row>
+    <row r="815">
+      <c r="A815" t="inlineStr">
+        <is>
+          <t>27/08/2026</t>
+        </is>
+      </c>
+      <c r="B815" t="n">
+        <v>22</v>
+      </c>
+      <c r="C815" t="inlineStr">
+        <is>
+          <t>làm sa bàn</t>
+        </is>
+      </c>
+      <c r="D815" t="n">
+        <v>4.6</v>
+      </c>
+      <c r="E815" t="n">
+        <v>1620</v>
+      </c>
+      <c r="F815" t="n">
+        <v>104</v>
+      </c>
+      <c r="G815" t="inlineStr">
+        <is>
+          <t>6.42%</t>
+        </is>
+      </c>
+      <c r="H815" t="inlineStr">
+        <is>
+          <t>https://mohinhkientruc.org/lam-sa-ban/</t>
+        </is>
+      </c>
+      <c r="I815" t="inlineStr">
+        <is>
+          <t>Standard Snippet</t>
+        </is>
+      </c>
+    </row>
+    <row r="816">
+      <c r="A816" t="inlineStr">
+        <is>
+          <t>28/08/2026</t>
+        </is>
+      </c>
+      <c r="B816" t="n">
+        <v>1</v>
+      </c>
+      <c r="C816" t="inlineStr">
+        <is>
+          <t>mô hình quy hoạch</t>
+        </is>
+      </c>
+      <c r="D816" t="n">
+        <v>7.5</v>
+      </c>
+      <c r="E816" t="n">
+        <v>50</v>
+      </c>
+      <c r="F816" t="n">
+        <v>4</v>
+      </c>
+      <c r="G816" t="inlineStr">
+        <is>
+          <t>8.00%</t>
+        </is>
+      </c>
+      <c r="H816" t="inlineStr">
+        <is>
+          <t>https://mohinhkientruc.org/danh-muc-du-an/mo-hinh-quy-hoach/</t>
+        </is>
+      </c>
+      <c r="I816" t="inlineStr">
+        <is>
+          <t>🖼️ Image Pack</t>
+        </is>
+      </c>
+    </row>
+    <row r="817">
+      <c r="A817" t="inlineStr">
+        <is>
+          <t>28/08/2026</t>
+        </is>
+      </c>
+      <c r="B817" t="n">
+        <v>2</v>
+      </c>
+      <c r="C817" t="inlineStr">
+        <is>
+          <t>mô hình kiến trúc</t>
+        </is>
+      </c>
+      <c r="D817" t="n">
+        <v>17.3</v>
+      </c>
+      <c r="E817" t="n">
+        <v>133</v>
+      </c>
+      <c r="F817" t="n">
+        <v>5</v>
+      </c>
+      <c r="G817" t="inlineStr">
+        <is>
+          <t>3.76%</t>
+        </is>
+      </c>
+      <c r="H817" t="inlineStr">
+        <is>
+          <t>https://mohinhkientruc.org/mo-hinh-kien-truc/</t>
+        </is>
+      </c>
+      <c r="I817" t="inlineStr">
+        <is>
+          <t>Standard Snippet</t>
+        </is>
+      </c>
+    </row>
+    <row r="818">
+      <c r="A818" t="inlineStr">
+        <is>
+          <t>28/08/2026</t>
+        </is>
+      </c>
+      <c r="B818" t="n">
+        <v>3</v>
+      </c>
+      <c r="C818" t="inlineStr">
+        <is>
+          <t>mô hình cao tầng</t>
+        </is>
+      </c>
+      <c r="D818" t="n">
+        <v>5</v>
+      </c>
+      <c r="E818" t="n">
+        <v>980</v>
+      </c>
+      <c r="F818" t="n">
+        <v>54</v>
+      </c>
+      <c r="G818" t="inlineStr">
+        <is>
+          <t>5.51%</t>
+        </is>
+      </c>
+      <c r="H818" t="inlineStr">
+        <is>
+          <t>https://mohinhkientruc.org/sa-ban-cao-tang/</t>
+        </is>
+      </c>
+      <c r="I818" t="inlineStr">
+        <is>
+          <t>Standard Snippet</t>
+        </is>
+      </c>
+    </row>
+    <row r="819">
+      <c r="A819" t="inlineStr">
+        <is>
+          <t>28/08/2026</t>
+        </is>
+      </c>
+      <c r="B819" t="n">
+        <v>4</v>
+      </c>
+      <c r="C819" t="inlineStr">
+        <is>
+          <t>mô hình nhà máy</t>
+        </is>
+      </c>
+      <c r="D819" t="n">
+        <v>6</v>
+      </c>
+      <c r="E819" t="n">
+        <v>1120</v>
+      </c>
+      <c r="F819" t="n">
+        <v>68</v>
+      </c>
+      <c r="G819" t="inlineStr">
+        <is>
+          <t>6.07%</t>
+        </is>
+      </c>
+      <c r="H819" t="inlineStr">
+        <is>
+          <t>https://mohinhkientruc.org/mo-hinh-nha-may/</t>
+        </is>
+      </c>
+      <c r="I819" t="inlineStr">
+        <is>
+          <t>Standard Snippet</t>
+        </is>
+      </c>
+    </row>
+    <row r="820">
+      <c r="A820" t="inlineStr">
+        <is>
+          <t>28/08/2026</t>
+        </is>
+      </c>
+      <c r="B820" t="n">
+        <v>5</v>
+      </c>
+      <c r="C820" t="inlineStr">
+        <is>
+          <t>mô hình thiết bị</t>
+        </is>
+      </c>
+      <c r="D820" t="n">
+        <v>9</v>
+      </c>
+      <c r="E820" t="n">
+        <v>640</v>
+      </c>
+      <c r="F820" t="n">
+        <v>25</v>
+      </c>
+      <c r="G820" t="inlineStr">
+        <is>
+          <t>3.91%</t>
+        </is>
+      </c>
+      <c r="H820" t="inlineStr">
+        <is>
+          <t>https://mohinhkientruc.org/mo-hinh-3d/</t>
+        </is>
+      </c>
+      <c r="I820" t="inlineStr">
+        <is>
+          <t>Standard Snippet</t>
+        </is>
+      </c>
+    </row>
+    <row r="821">
+      <c r="A821" t="inlineStr">
+        <is>
+          <t>28/08/2026</t>
+        </is>
+      </c>
+      <c r="B821" t="n">
+        <v>6</v>
+      </c>
+      <c r="C821" t="inlineStr">
+        <is>
+          <t>mô hình trường học</t>
+        </is>
+      </c>
+      <c r="D821" t="n">
+        <v>7</v>
+      </c>
+      <c r="E821" t="n">
+        <v>720</v>
+      </c>
+      <c r="F821" t="n">
+        <v>38</v>
+      </c>
+      <c r="G821" t="inlineStr">
+        <is>
+          <t>5.28%</t>
+        </is>
+      </c>
+      <c r="H821" t="inlineStr">
+        <is>
+          <t>https://mohinhkientruc.org/lam-sa-ban-truong-hoc/</t>
+        </is>
+      </c>
+      <c r="I821" t="inlineStr">
+        <is>
+          <t>Standard Snippet</t>
+        </is>
+      </c>
+    </row>
+    <row r="822">
+      <c r="A822" t="inlineStr">
+        <is>
+          <t>28/08/2026</t>
+        </is>
+      </c>
+      <c r="B822" t="n">
+        <v>7</v>
+      </c>
+      <c r="C822" t="inlineStr">
+        <is>
+          <t>mô hình bệnh viện</t>
+        </is>
+      </c>
+      <c r="D822" t="n">
+        <v>8</v>
+      </c>
+      <c r="E822" t="n">
+        <v>530</v>
+      </c>
+      <c r="F822" t="n">
+        <v>22</v>
+      </c>
+      <c r="G822" t="inlineStr">
+        <is>
+          <t>4.15%</t>
+        </is>
+      </c>
+      <c r="H822" t="inlineStr">
+        <is>
+          <t>https://mohinhkientruc.org/mo-hinh-tod-sa-ban/</t>
+        </is>
+      </c>
+      <c r="I822" t="inlineStr">
+        <is>
+          <t>Standard Snippet</t>
+        </is>
+      </c>
+    </row>
+    <row r="823">
+      <c r="A823" t="inlineStr">
+        <is>
+          <t>28/08/2026</t>
+        </is>
+      </c>
+      <c r="B823" t="n">
+        <v>8</v>
+      </c>
+      <c r="C823" t="inlineStr">
+        <is>
+          <t>sa bàn quy hoạch</t>
+        </is>
+      </c>
+      <c r="D823" t="n">
+        <v>4</v>
+      </c>
+      <c r="E823" t="n">
+        <v>1650</v>
+      </c>
+      <c r="F823" t="n">
+        <v>118</v>
+      </c>
+      <c r="G823" t="inlineStr">
+        <is>
+          <t>7.15%</t>
+        </is>
+      </c>
+      <c r="H823" t="inlineStr">
+        <is>
+          <t>https://mohinhkientruc.org/dich-vu-lam-sa-ban-quy-hoach/</t>
+        </is>
+      </c>
+      <c r="I823" t="inlineStr">
+        <is>
+          <t>🖼️ Image Pack</t>
+        </is>
+      </c>
+    </row>
+    <row r="824">
+      <c r="A824" t="inlineStr">
+        <is>
+          <t>28/08/2026</t>
+        </is>
+      </c>
+      <c r="B824" t="n">
+        <v>9</v>
+      </c>
+      <c r="C824" t="inlineStr">
+        <is>
+          <t>sa bàn kiến trúc</t>
+        </is>
+      </c>
+      <c r="D824" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="E824" t="n">
+        <v>2100</v>
+      </c>
+      <c r="F824" t="n">
+        <v>135</v>
+      </c>
+      <c r="G824" t="inlineStr">
+        <is>
+          <t>6.43%</t>
+        </is>
+      </c>
+      <c r="H824" t="inlineStr">
+        <is>
+          <t>https://mohinhkientruc.org/sa-ban-kien-truc/</t>
+        </is>
+      </c>
+      <c r="I824" t="inlineStr">
+        <is>
+          <t>Standard Snippet</t>
+        </is>
+      </c>
+    </row>
+    <row r="825">
+      <c r="A825" t="inlineStr">
+        <is>
+          <t>28/08/2026</t>
+        </is>
+      </c>
+      <c r="B825" t="n">
+        <v>10</v>
+      </c>
+      <c r="C825" t="inlineStr">
+        <is>
+          <t>sa bàn cao tầng</t>
+        </is>
+      </c>
+      <c r="D825" t="n">
+        <v>5.5</v>
+      </c>
+      <c r="E825" t="n">
+        <v>870</v>
+      </c>
+      <c r="F825" t="n">
+        <v>46</v>
+      </c>
+      <c r="G825" t="inlineStr">
+        <is>
+          <t>5.29%</t>
+        </is>
+      </c>
+      <c r="H825" t="inlineStr">
+        <is>
+          <t>https://mohinhkientruc.org/sa-ban-cao-tang/</t>
+        </is>
+      </c>
+      <c r="I825" t="inlineStr">
+        <is>
+          <t>Standard Snippet</t>
+        </is>
+      </c>
+    </row>
+    <row r="826">
+      <c r="A826" t="inlineStr">
+        <is>
+          <t>28/08/2026</t>
+        </is>
+      </c>
+      <c r="B826" t="n">
+        <v>11</v>
+      </c>
+      <c r="C826" t="inlineStr">
+        <is>
+          <t>sa bàn nhà máy</t>
+        </is>
+      </c>
+      <c r="D826" t="n">
+        <v>2.2</v>
+      </c>
+      <c r="E826" t="n">
+        <v>11</v>
+      </c>
+      <c r="F826" t="n">
+        <v>1</v>
+      </c>
+      <c r="G826" t="inlineStr">
+        <is>
+          <t>9.09%</t>
+        </is>
+      </c>
+      <c r="H826" t="inlineStr">
+        <is>
+          <t>https://mohinhkientruc.org/thi-cong-sa-ban-nha-may-khu-cong-nghiep/</t>
+        </is>
+      </c>
+      <c r="I826" t="inlineStr">
+        <is>
+          <t>Standard Snippet</t>
+        </is>
+      </c>
+    </row>
+    <row r="827">
+      <c r="A827" t="inlineStr">
+        <is>
+          <t>28/08/2026</t>
+        </is>
+      </c>
+      <c r="B827" t="n">
+        <v>12</v>
+      </c>
+      <c r="C827" t="inlineStr">
+        <is>
+          <t>sa bàn thiết bị</t>
+        </is>
+      </c>
+      <c r="D827" t="n">
+        <v>9.5</v>
+      </c>
+      <c r="E827" t="n">
+        <v>480</v>
+      </c>
+      <c r="F827" t="n">
+        <v>18</v>
+      </c>
+      <c r="G827" t="inlineStr">
+        <is>
+          <t>3.75%</t>
+        </is>
+      </c>
+      <c r="H827" t="inlineStr">
+        <is>
+          <t>https://mohinhkientruc.org/sa-ban-noi-that/</t>
+        </is>
+      </c>
+      <c r="I827" t="inlineStr">
+        <is>
+          <t>Standard Snippet</t>
+        </is>
+      </c>
+    </row>
+    <row r="828">
+      <c r="A828" t="inlineStr">
+        <is>
+          <t>28/08/2026</t>
+        </is>
+      </c>
+      <c r="B828" t="n">
+        <v>13</v>
+      </c>
+      <c r="C828" t="inlineStr">
+        <is>
+          <t>sa bàn trường học</t>
+        </is>
+      </c>
+      <c r="D828" t="n">
+        <v>6.7</v>
+      </c>
+      <c r="E828" t="n">
+        <v>3</v>
+      </c>
+      <c r="F828" t="n">
+        <v>1</v>
+      </c>
+      <c r="G828" t="inlineStr">
+        <is>
+          <t>33.33%</t>
+        </is>
+      </c>
+      <c r="H828" t="inlineStr">
+        <is>
+          <t>https://mohinhkientruc.org/lam-sa-ban-truong-hoc/</t>
+        </is>
+      </c>
+      <c r="I828" t="inlineStr">
+        <is>
+          <t>Standard Snippet</t>
+        </is>
+      </c>
+    </row>
+    <row r="829">
+      <c r="A829" t="inlineStr">
+        <is>
+          <t>28/08/2026</t>
+        </is>
+      </c>
+      <c r="B829" t="n">
+        <v>14</v>
+      </c>
+      <c r="C829" t="inlineStr">
+        <is>
+          <t>sa bàn bệnh viện</t>
+        </is>
+      </c>
+      <c r="D829" t="n">
+        <v>8.5</v>
+      </c>
+      <c r="E829" t="n">
+        <v>590</v>
+      </c>
+      <c r="F829" t="n">
+        <v>26</v>
+      </c>
+      <c r="G829" t="inlineStr">
+        <is>
+          <t>4.41%</t>
+        </is>
+      </c>
+      <c r="H829" t="inlineStr">
+        <is>
+          <t>https://mohinhkientruc.org/du-an-noi-bat/</t>
+        </is>
+      </c>
+      <c r="I829" t="inlineStr">
+        <is>
+          <t>Standard Snippet</t>
+        </is>
+      </c>
+    </row>
+    <row r="830">
+      <c r="A830" t="inlineStr">
+        <is>
+          <t>28/08/2026</t>
+        </is>
+      </c>
+      <c r="B830" t="n">
+        <v>15</v>
+      </c>
+      <c r="C830" t="inlineStr">
+        <is>
+          <t>vận chuyển mô hình</t>
+        </is>
+      </c>
+      <c r="D830" t="n">
+        <v>6.8</v>
+      </c>
+      <c r="E830" t="n">
+        <v>820</v>
+      </c>
+      <c r="F830" t="n">
+        <v>45</v>
+      </c>
+      <c r="G830" t="inlineStr">
+        <is>
+          <t>5.49%</t>
+        </is>
+      </c>
+      <c r="H830" t="inlineStr">
+        <is>
+          <t>https://mohinhkientruc.org/van-chuyen-sa-ban-kien-truc/</t>
+        </is>
+      </c>
+      <c r="I830" t="inlineStr">
+        <is>
+          <t>Standard Snippet</t>
+        </is>
+      </c>
+    </row>
+    <row r="831">
+      <c r="A831" t="inlineStr">
+        <is>
+          <t>28/08/2026</t>
+        </is>
+      </c>
+      <c r="B831" t="n">
+        <v>16</v>
+      </c>
+      <c r="C831" t="inlineStr">
+        <is>
+          <t>vận chuyển sa bàn</t>
+        </is>
+      </c>
+      <c r="D831" t="n">
+        <v>7.2</v>
+      </c>
+      <c r="E831" t="n">
+        <v>760</v>
+      </c>
+      <c r="F831" t="n">
+        <v>38</v>
+      </c>
+      <c r="G831" t="inlineStr">
+        <is>
+          <t>5.00%</t>
+        </is>
+      </c>
+      <c r="H831" t="inlineStr">
+        <is>
+          <t>https://mohinhkientruc.org/van-chuyen-sa-ban-kien-truc/</t>
+        </is>
+      </c>
+      <c r="I831" t="inlineStr">
+        <is>
+          <t>Standard Snippet</t>
+        </is>
+      </c>
+    </row>
+    <row r="832">
+      <c r="A832" t="inlineStr">
+        <is>
+          <t>28/08/2026</t>
+        </is>
+      </c>
+      <c r="B832" t="n">
+        <v>17</v>
+      </c>
+      <c r="C832" t="inlineStr">
+        <is>
+          <t>sửa chữa mô hình</t>
+        </is>
+      </c>
+      <c r="D832" t="n">
+        <v>5.4</v>
+      </c>
+      <c r="E832" t="n">
+        <v>930</v>
+      </c>
+      <c r="F832" t="n">
+        <v>58</v>
+      </c>
+      <c r="G832" t="inlineStr">
+        <is>
+          <t>6.24%</t>
+        </is>
+      </c>
+      <c r="H832" t="inlineStr">
+        <is>
+          <t>https://mohinhkientruc.org/sua-chua-mo-hinh-kien-truc/</t>
+        </is>
+      </c>
+      <c r="I832" t="inlineStr">
+        <is>
+          <t>Standard Snippet</t>
+        </is>
+      </c>
+    </row>
+    <row r="833">
+      <c r="A833" t="inlineStr">
+        <is>
+          <t>28/08/2026</t>
+        </is>
+      </c>
+      <c r="B833" t="n">
+        <v>18</v>
+      </c>
+      <c r="C833" t="inlineStr">
+        <is>
+          <t>sửa chữa sa bàn</t>
+        </is>
+      </c>
+      <c r="D833" t="n">
+        <v>5.8</v>
+      </c>
+      <c r="E833" t="n">
+        <v>880</v>
+      </c>
+      <c r="F833" t="n">
+        <v>52</v>
+      </c>
+      <c r="G833" t="inlineStr">
+        <is>
+          <t>5.91%</t>
+        </is>
+      </c>
+      <c r="H833" t="inlineStr">
+        <is>
+          <t>https://mohinhkientruc.org/sua-chua-mo-hinh-kien-truc/</t>
+        </is>
+      </c>
+      <c r="I833" t="inlineStr">
+        <is>
+          <t>Standard Snippet</t>
+        </is>
+      </c>
+    </row>
+    <row r="834">
+      <c r="A834" t="inlineStr">
+        <is>
+          <t>28/08/2026</t>
+        </is>
+      </c>
+      <c r="B834" t="n">
+        <v>19</v>
+      </c>
+      <c r="C834" t="inlineStr">
+        <is>
+          <t>công ty mô hình kiến trúc</t>
+        </is>
+      </c>
+      <c r="D834" t="n">
+        <v>41.7</v>
+      </c>
+      <c r="E834" t="n">
+        <v>34</v>
+      </c>
+      <c r="F834" t="n">
+        <v>0</v>
+      </c>
+      <c r="G834" t="inlineStr">
+        <is>
+          <t>0.00%</t>
+        </is>
+      </c>
+      <c r="H834" t="inlineStr">
+        <is>
+          <t>https://mohinhkientruc.org/cong-ty-lam-mo-hinh/</t>
+        </is>
+      </c>
+      <c r="I834" t="inlineStr">
+        <is>
+          <t>🖼️ Image Pack</t>
+        </is>
+      </c>
+    </row>
+    <row r="835">
+      <c r="A835" t="inlineStr">
+        <is>
+          <t>28/08/2026</t>
+        </is>
+      </c>
+      <c r="B835" t="n">
+        <v>20</v>
+      </c>
+      <c r="C835" t="inlineStr">
+        <is>
+          <t>công ty sa bàn kiến trúc</t>
+        </is>
+      </c>
+      <c r="D835" t="n">
+        <v>3.2</v>
+      </c>
+      <c r="E835" t="n">
+        <v>2410</v>
+      </c>
+      <c r="F835" t="n">
+        <v>168</v>
+      </c>
+      <c r="G835" t="inlineStr">
+        <is>
+          <t>6.97%</t>
+        </is>
+      </c>
+      <c r="H835" t="inlineStr">
+        <is>
+          <t>https://mohinhkientruc.org/</t>
+        </is>
+      </c>
+      <c r="I835" t="inlineStr">
+        <is>
+          <t>Standard Snippet</t>
+        </is>
+      </c>
+    </row>
+    <row r="836">
+      <c r="A836" t="inlineStr">
+        <is>
+          <t>28/08/2026</t>
+        </is>
+      </c>
+      <c r="B836" t="n">
+        <v>21</v>
+      </c>
+      <c r="C836" t="inlineStr">
+        <is>
+          <t>làm mô hình</t>
+        </is>
+      </c>
+      <c r="D836" t="n">
+        <v>4.2</v>
+      </c>
+      <c r="E836" t="n">
+        <v>1780</v>
+      </c>
+      <c r="F836" t="n">
+        <v>121</v>
+      </c>
+      <c r="G836" t="inlineStr">
+        <is>
+          <t>6.80%</t>
+        </is>
+      </c>
+      <c r="H836" t="inlineStr">
+        <is>
+          <t>https://mohinhkientruc.org/lam-mo-hinh-kien-truc/</t>
+        </is>
+      </c>
+      <c r="I836" t="inlineStr">
+        <is>
+          <t>Standard Snippet</t>
+        </is>
+      </c>
+    </row>
+    <row r="837">
+      <c r="A837" t="inlineStr">
+        <is>
+          <t>28/08/2026</t>
+        </is>
+      </c>
+      <c r="B837" t="n">
+        <v>22</v>
+      </c>
+      <c r="C837" t="inlineStr">
+        <is>
+          <t>làm sa bàn</t>
+        </is>
+      </c>
+      <c r="D837" t="n">
+        <v>4.6</v>
+      </c>
+      <c r="E837" t="n">
+        <v>1620</v>
+      </c>
+      <c r="F837" t="n">
+        <v>104</v>
+      </c>
+      <c r="G837" t="inlineStr">
+        <is>
+          <t>6.42%</t>
+        </is>
+      </c>
+      <c r="H837" t="inlineStr">
+        <is>
+          <t>https://mohinhkientruc.org/lam-sa-ban/</t>
+        </is>
+      </c>
+      <c r="I837" t="inlineStr">
+        <is>
+          <t>Standard Snippet</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>